<commit_message>
Plantilla diseño ETL excel
</commit_message>
<xml_diff>
--- a/Segundo entregable/PlantillaDisenioETL.xlsx
+++ b/Segundo entregable/PlantillaDisenioETL.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Profesor\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Documents\GitHub\entrega_proyecto_MIAD_modelado_datos\Segundo entregable\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BA3F12E-9188-4992-AA38-49C18921EADF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12030"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PlantillaDiseñoETL" sheetId="1" r:id="rId1"/>
@@ -25,20 +26,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="15">
-  <si>
-    <t>NOMBRE ENTIDAD</t>
-  </si>
-  <si>
-    <t>* NombreFuente</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="52">
   <si>
     <t>Campos a incluir:</t>
   </si>
   <si>
-    <t>* NombreCampo1</t>
-  </si>
-  <si>
     <t>*…</t>
   </si>
   <si>
@@ -58,9 +50,6 @@
   </si>
   <si>
     <t>Destino de los datos:</t>
-  </si>
-  <si>
-    <t>* NombreDestino</t>
   </si>
   <si>
     <t>Campos a cargar:</t>
@@ -81,15 +70,138 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>NOMBREPROYECTO</t>
+      <t>PROYECTO RaSA</t>
     </r>
+  </si>
+  <si>
+    <t>DimFecha</t>
+  </si>
+  <si>
+    <t>* FuentePlanesBeneficio_Copia_E</t>
+  </si>
+  <si>
+    <t>* Fecha</t>
+  </si>
+  <si>
+    <t>* DimFecha</t>
+  </si>
+  <si>
+    <t>* SK_Fecha</t>
+  </si>
+  <si>
+    <t>* Año</t>
+  </si>
+  <si>
+    <t>* Trimestre</t>
+  </si>
+  <si>
+    <t>* Mes</t>
+  </si>
+  <si>
+    <t>* NombreMes</t>
+  </si>
+  <si>
+    <t>* Día</t>
+  </si>
+  <si>
+    <t>DimProveedor</t>
+  </si>
+  <si>
+    <t>* idProveedor_T</t>
+  </si>
+  <si>
+    <t>* idPlan_T</t>
+  </si>
+  <si>
+    <t>* idTipoBeneficio_T</t>
+  </si>
+  <si>
+    <t>* idAreaDeServicio_T</t>
+  </si>
+  <si>
+    <t>* idCondicionesDePagoCopago_T</t>
+  </si>
+  <si>
+    <t>* idCondicionesDePagoCoseguro_T</t>
+  </si>
+  <si>
+    <t>* idNivelServicio_T</t>
+  </si>
+  <si>
+    <t>* valorCopago</t>
+  </si>
+  <si>
+    <t>* valorCoseguro</t>
+  </si>
+  <si>
+    <t>* cantidadLimite</t>
+  </si>
+  <si>
+    <t>* DimProveedor</t>
+  </si>
+  <si>
+    <t>* SK_Proveedor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">* idProveedor_T </t>
+  </si>
+  <si>
+    <t>DimPlan</t>
+  </si>
+  <si>
+    <t>* DimPlan</t>
+  </si>
+  <si>
+    <t>* SK_Plan</t>
+  </si>
+  <si>
+    <t>DimCondicionPago</t>
+  </si>
+  <si>
+    <t>* FuenteTiposBeneficio_Copia_E</t>
+  </si>
+  <si>
+    <t>* idCondicionesDePago_T</t>
+  </si>
+  <si>
+    <t>* FuenteCondicionesPago_Copia_E</t>
+  </si>
+  <si>
+    <t>* Descripcion</t>
+  </si>
+  <si>
+    <t>* Nombre</t>
+  </si>
+  <si>
+    <t>* UnidadDelLimite</t>
+  </si>
+  <si>
+    <t>* EsEHB</t>
+  </si>
+  <si>
+    <t>* EstaCubiertoPorSeguro</t>
+  </si>
+  <si>
+    <t>* TieneLimiteCuantitativo</t>
+  </si>
+  <si>
+    <t>* ExcluidoDelDesembolsoMaximoDentroDeLaRed</t>
+  </si>
+  <si>
+    <t>* ExcluidoDelDesembolsoMaximoFueraDeLaRed</t>
+  </si>
+  <si>
+    <t>* DimCondicionPago</t>
+  </si>
+  <si>
+    <t>* Tipo</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -123,6 +235,13 @@
     <font>
       <b/>
       <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -163,10 +282,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -184,9 +304,14 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{7687CB3D-81DF-4C88-A1B3-5BED9B84F9B2}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -212,25 +337,31 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>790575</xdr:colOff>
+      <xdr:colOff>472441</xdr:colOff>
       <xdr:row>6</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>2552700</xdr:colOff>
+      <xdr:colOff>2887981</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="Rectángulo redondeado 1"/>
+        <xdr:cNvPr id="2" name="Rectángulo redondeado 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5705475" y="1295400"/>
-          <a:ext cx="1762125" cy="323850"/>
+          <a:off x="3916681" y="1249680"/>
+          <a:ext cx="2415540" cy="308610"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -266,7 +397,7 @@
                 <a:srgbClr val="FF0000"/>
               </a:solidFill>
             </a:rPr>
-            <a:t>Fuente de datos</a:t>
+            <a:t>FuentePlanesBeneficio_Copia_E</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -275,28 +406,34 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>1781175</xdr:colOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>15240</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>104775</xdr:rowOff>
+      <xdr:rowOff>121920</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>790575</xdr:colOff>
+      <xdr:colOff>472441</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="4" name="Conector recto de flecha 3"/>
+        <xdr:cNvPr id="4" name="Conector recto de flecha 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvCxnSpPr>
           <a:stCxn id="2" idx="1"/>
         </xdr:cNvCxnSpPr>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1" flipV="1">
-          <a:off x="4124325" y="1438275"/>
-          <a:ext cx="1581150" cy="19050"/>
+          <a:off x="2667000" y="1402080"/>
+          <a:ext cx="1249681" cy="1905"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -337,7 +474,13 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="7" name="Rectángulo redondeado 6"/>
+        <xdr:cNvPr id="7" name="Rectángulo redondeado 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000007000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -374,7 +517,7 @@
                 <a:srgbClr val="FF0000"/>
               </a:solidFill>
             </a:rPr>
-            <a:t>T1. Descripción detallada</a:t>
+            <a:t>T1. Eliminar fechas nulas.</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -384,25 +527,31 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>809625</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:colOff>548640</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>99060</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>2571750</xdr:colOff>
+      <xdr:colOff>3413759</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>171450</xdr:rowOff>
+      <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="8" name="Rectángulo redondeado 7"/>
+        <xdr:cNvPr id="8" name="Rectángulo redondeado 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000008000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5724525" y="3657600"/>
-          <a:ext cx="1762125" cy="323850"/>
+          <a:off x="4076700" y="3208020"/>
+          <a:ext cx="2865119" cy="525780"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -433,7 +582,7 @@
                 <a:srgbClr val="FF0000"/>
               </a:solidFill>
             </a:rPr>
-            <a:t>Tn. Descripción detallada</a:t>
+            <a:t>T3. Convertir todas las fechas al mismo formato. YYYY-MM-DD</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -443,27 +592,33 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1671638</xdr:colOff>
+      <xdr:colOff>1676401</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1676400</xdr:colOff>
+      <xdr:colOff>1680211</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="9" name="Conector recto de flecha 8"/>
+        <xdr:cNvPr id="9" name="Conector recto de flecha 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000009000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvCxnSpPr>
           <a:stCxn id="2" idx="2"/>
         </xdr:cNvCxnSpPr>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6586538" y="1619250"/>
-          <a:ext cx="4762" cy="514350"/>
+        <a:xfrm flipH="1">
+          <a:off x="5120641" y="1558290"/>
+          <a:ext cx="3810" cy="491490"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -498,19 +653,25 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>2571750</xdr:colOff>
+      <xdr:colOff>2926080</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="12" name="Rectángulo redondeado 11"/>
+        <xdr:cNvPr id="12" name="Rectángulo redondeado 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000C000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5724525" y="2914650"/>
-          <a:ext cx="1762125" cy="323850"/>
+          <a:off x="4337685" y="2800350"/>
+          <a:ext cx="2116455" cy="308610"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -541,7 +702,7 @@
                 <a:srgbClr val="FF0000"/>
               </a:solidFill>
             </a:rPr>
-            <a:t>T2. Descripción detallada</a:t>
+            <a:t>T2. Eliminar fechas duplicadas.</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -551,25 +712,31 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>790575</xdr:colOff>
+      <xdr:colOff>579120</xdr:colOff>
       <xdr:row>6</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>2552700</xdr:colOff>
+      <xdr:colOff>2781300</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="16" name="Rectángulo redondeado 15"/>
+        <xdr:cNvPr id="16" name="Rectángulo redondeado 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000010000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5705475" y="1295400"/>
-          <a:ext cx="1762125" cy="323850"/>
+          <a:off x="10767060" y="1249680"/>
+          <a:ext cx="2202180" cy="308610"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -605,7 +772,7 @@
                 <a:srgbClr val="FF0000"/>
               </a:solidFill>
             </a:rPr>
-            <a:t>Fuente de datos</a:t>
+            <a:t>FuentePlanesBeneficio_Copia_E</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -615,27 +782,33 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>1781175</xdr:colOff>
+      <xdr:colOff>1377316</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>104775</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>790575</xdr:colOff>
+      <xdr:colOff>579120</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="17" name="Conector recto de flecha 16"/>
+        <xdr:cNvPr id="17" name="Conector recto de flecha 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000011000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvCxnSpPr>
           <a:stCxn id="16" idx="1"/>
         </xdr:cNvCxnSpPr>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1" flipV="1">
-          <a:off x="4124325" y="1438275"/>
-          <a:ext cx="1581150" cy="19050"/>
+          <a:off x="9393556" y="1384935"/>
+          <a:ext cx="1373504" cy="19050"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -664,25 +837,31 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>790575</xdr:colOff>
+      <xdr:colOff>175260</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>2552700</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
+      <xdr:colOff>3032759</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="18" name="Rectángulo redondeado 17"/>
+        <xdr:cNvPr id="18" name="Rectángulo redondeado 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000012000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5705475" y="2438400"/>
-          <a:ext cx="1762125" cy="323850"/>
+          <a:off x="10980420" y="2346960"/>
+          <a:ext cx="2857499" cy="723900"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -713,8 +892,21 @@
                 <a:srgbClr val="FF0000"/>
               </a:solidFill>
             </a:rPr>
-            <a:t>T1. Descripción detallada</a:t>
-          </a:r>
+            <a:t>T1. </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Validación de datos obligatorios: Eliminar registros cuyo idProveedor_T sea nulo o vacío.</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-CO" sz="1100" b="0">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </a:endParaRPr>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -723,86 +915,33 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>809625</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>2571750</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>171450</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="19" name="Rectángulo redondeado 18"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5724525" y="3657600"/>
-          <a:ext cx="1762125" cy="323850"/>
-        </a:xfrm>
-        <a:prstGeom prst="roundRect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent6"/>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="lt1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent6"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="es-CO" sz="1100">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Tn. Descripción detallada</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>1671638</xdr:colOff>
+      <xdr:colOff>1676400</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>1676400</xdr:colOff>
+      <xdr:colOff>1680210</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="20" name="Conector recto de flecha 19"/>
+        <xdr:cNvPr id="20" name="Conector recto de flecha 19">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000014000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvCxnSpPr>
           <a:stCxn id="16" idx="2"/>
         </xdr:cNvCxnSpPr>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6586538" y="1619250"/>
-          <a:ext cx="4762" cy="514350"/>
+        <a:xfrm flipH="1">
+          <a:off x="11864340" y="1558290"/>
+          <a:ext cx="3810" cy="491490"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -830,85 +969,32 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>809625</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>2571750</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="21" name="Rectángulo redondeado 20"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5724525" y="2914650"/>
-          <a:ext cx="1762125" cy="323850"/>
-        </a:xfrm>
-        <a:prstGeom prst="roundRect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent6"/>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="lt1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent6"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="es-CO" sz="1100">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>T2. Descripción detallada</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>790575</xdr:colOff>
+      <xdr:colOff>464821</xdr:colOff>
       <xdr:row>6</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>2552700</xdr:colOff>
+      <xdr:colOff>2903221</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="22" name="Rectángulo redondeado 21"/>
+        <xdr:cNvPr id="22" name="Rectángulo redondeado 21">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000016000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5705475" y="1295400"/>
-          <a:ext cx="1762125" cy="323850"/>
+          <a:off x="17823181" y="1249680"/>
+          <a:ext cx="2438400" cy="308610"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -944,7 +1030,7 @@
                 <a:srgbClr val="FF0000"/>
               </a:solidFill>
             </a:rPr>
-            <a:t>Fuente de datos</a:t>
+            <a:t>FuentePlanesBeneficio_Copia_E</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -953,28 +1039,34 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>1781175</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>7620</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>104775</xdr:rowOff>
+      <xdr:rowOff>123825</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>790575</xdr:colOff>
+      <xdr:colOff>464821</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
+      <xdr:rowOff>137160</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="23" name="Conector recto de flecha 22"/>
+        <xdr:cNvPr id="23" name="Conector recto de flecha 22">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000017000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvCxnSpPr>
           <a:stCxn id="22" idx="1"/>
         </xdr:cNvCxnSpPr>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
-        <a:xfrm flipH="1" flipV="1">
-          <a:off x="4124325" y="1438275"/>
-          <a:ext cx="1581150" cy="19050"/>
+        <a:xfrm flipH="1">
+          <a:off x="16573500" y="1403985"/>
+          <a:ext cx="1249681" cy="13335"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -1003,145 +1095,33 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>790575</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>2552700</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="24" name="Rectángulo redondeado 23"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5705475" y="2438400"/>
-          <a:ext cx="1762125" cy="323850"/>
-        </a:xfrm>
-        <a:prstGeom prst="roundRect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent6"/>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="lt1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent6"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="es-CO" sz="1100">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>T1. Descripción detallada</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>809625</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>2571750</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>171450</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="25" name="Rectángulo redondeado 24"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5724525" y="3657600"/>
-          <a:ext cx="1762125" cy="323850"/>
-        </a:xfrm>
-        <a:prstGeom prst="roundRect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent6"/>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="lt1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent6"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="es-CO" sz="1100">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Tn. Descripción detallada</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>1671638</xdr:colOff>
+      <xdr:colOff>1676401</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>1676400</xdr:colOff>
+      <xdr:colOff>1684021</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="26" name="Conector recto de flecha 25"/>
+        <xdr:cNvPr id="26" name="Conector recto de flecha 25">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00001A000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvCxnSpPr>
           <a:stCxn id="22" idx="2"/>
         </xdr:cNvCxnSpPr>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6586538" y="1619250"/>
-          <a:ext cx="4762" cy="514350"/>
+        <a:xfrm flipH="1">
+          <a:off x="19034761" y="1558290"/>
+          <a:ext cx="7620" cy="491490"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -1169,26 +1149,32 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>809625</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>106680</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>121920</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>2571750</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>3611880</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>106680</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="27" name="Rectángulo redondeado 26"/>
+        <xdr:cNvPr id="28" name="Rectángulo redondeado 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8598D1B5-FB4E-48A3-9892-6F4C9C647A45}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5724525" y="2914650"/>
-          <a:ext cx="1762125" cy="323850"/>
+          <a:off x="3634740" y="3779520"/>
+          <a:ext cx="3505200" cy="1264920"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -1219,8 +1205,1566 @@
                 <a:srgbClr val="FF0000"/>
               </a:solidFill>
             </a:rPr>
-            <a:t>T2. Descripción detallada</a:t>
-          </a:r>
+            <a:t>T4. Generar automáticamente los atributos del calendario.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>A partir de cada fecha obtener: Año,</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t> S</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>emestre, Trimestre,</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Mes, Nombre del mes, </a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Día,</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Día de la semana (opcional) </a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Número de semana (opcional)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:endParaRPr lang="es-CO" sz="1100">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>882015</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>175260</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>2887980</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>118110</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="29" name="Rectángulo redondeado 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B6F6C4F1-7250-411B-BF78-DBAC30045137}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4410075" y="5113020"/>
+          <a:ext cx="2005965" cy="308610"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T5. Generar la clave sustituta.</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>207645</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>34290</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>3002280</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="37" name="Rectángulo redondeado 20">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D467B801-86C9-4CEF-B62F-24139C84D806}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11012805" y="3143250"/>
+          <a:ext cx="2794635" cy="1070610"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T2. Eliminación de duplicados: </a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Un mismo proveedor puede aparecer asociado a muchos planes.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Se debe obtener únicamente un registro por cada ID_Proveedor.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>200025</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>118110</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>2994660</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>137160</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="40" name="Rectángulo redondeado 20">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A040BA59-62C2-4AA1-9DC7-049DCC56B341}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11005185" y="4324350"/>
+          <a:ext cx="2794635" cy="750570"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T3. </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Normalización</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>: </a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Si existen espacios en blanco al inicio o final del identificador, eliminarlos.</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>192405</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>2987040</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="41" name="Rectángulo redondeado 20">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EAFE4F4F-4E53-49B1-AA7E-FD877A4EF2D7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10997565" y="5139690"/>
+          <a:ext cx="2794635" cy="1078230"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T4. </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Generación de clave sustituta: Crear</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>SK_Proveedor</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>como llave primaria de la dimensión.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>El idProveedor_T permanece como clave natural.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:endParaRPr lang="es-CO" sz="1100">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>207645</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>3002280</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>137160</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="42" name="Rectángulo redondeado 20">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DB2875B2-B7A2-41A1-8184-7B75CE359E98}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11012805" y="6313170"/>
+          <a:ext cx="2794635" cy="956310"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T5. </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Validación de unicidad: Verificar que no existan dos registros con el mismo ID_Proveedor después de la transformación.</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-CO" sz="1100">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>129540</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>3497580</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>99060</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="48" name="Rectángulo redondeado 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{139B8776-A481-4277-8B6B-CEF108145F0F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17716500" y="2308860"/>
+          <a:ext cx="3368040" cy="350520"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T1. </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Eliminar planes con identificador nulo.</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-CO" sz="1100" b="0">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>129540</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>3497580</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="49" name="Rectángulo redondeado 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D1B7B288-3815-45B8-8C91-F803811B659F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17716500" y="2743200"/>
+          <a:ext cx="3368040" cy="350520"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T2. </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Eliminar registros duplicados.</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-CO" sz="1100" b="0">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>3482340</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="50" name="Rectángulo redondeado 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B036BB6D-B1FA-4741-B308-8DFDDBFFBE5A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17701260" y="3169920"/>
+          <a:ext cx="3368040" cy="487680"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T3. </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Normalizar el identificador del plan (eliminar espacios, caracteres no válidos si aplica).</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-CO" sz="1100" b="0">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>137160</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>53340</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>3520440</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="51" name="Rectángulo redondeado 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F320024D-BD75-4EA1-9674-8578456BF850}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17724120" y="3710940"/>
+          <a:ext cx="3383280" cy="358140"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T4. </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Generar SK_Plan como clave sustituta.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:endParaRPr lang="es-CO" sz="1100" b="0">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>144780</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>129540</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>3505200</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>121920</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="52" name="Rectángulo redondeado 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{34E23C8A-E962-4576-AF8F-60528A13CA4D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17731740" y="4152900"/>
+          <a:ext cx="3360420" cy="358140"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T5</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>. Validar unicidad. </a:t>
+          </a:r>
+          <a:endParaRPr lang="es-CO" sz="1100" b="0">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>464821</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>2903221</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>140970</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="53" name="Rectángulo redondeado 21">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1C54793A-9031-4A20-920B-D81142EB0E0D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="25435561" y="1112520"/>
+          <a:ext cx="2438400" cy="491490"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="CCCCFF"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>FuenteCondicionesPago_Copia_E</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>FuenteTiposBeneficio_Copia_E</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>464821</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>78105</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="54" name="Conector recto de flecha 53">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0716A02A-5415-4F16-B3A4-D7811D92598A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="53" idx="1"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1" flipV="1">
+          <a:off x="24178260" y="1356360"/>
+          <a:ext cx="1257301" cy="1905"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>1684020</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>140970</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>1684021</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="55" name="Conector recto de flecha 54">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F2EC10F3-DE4C-475D-89FA-2EF2BF0A6D5D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="53" idx="2"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="26654760" y="1604010"/>
+          <a:ext cx="1" cy="392430"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>83820</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>3093720</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="56" name="Rectángulo redondeado 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8D476CBF-8D74-4235-B060-ECE17FF9DE0C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="25679400" y="2308860"/>
+          <a:ext cx="3009900" cy="693420"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T1. </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Validación de obligatoriedad: Eliminar registros cuyo identificador de condición sea nulo. </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" b="0" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:endParaRPr lang="es-CO" sz="1100" b="0">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>3086100</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="57" name="Rectángulo redondeado 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E4825CA5-B42D-4928-B779-B2F8ED96788A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="25671780" y="3070860"/>
+          <a:ext cx="3009900" cy="480060"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T2. </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Eliminación de duplicados: Conservar un único registro por condición de pago.</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-CO" sz="1100" b="0">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>68580</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>3093720</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>129540</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="58" name="Rectángulo redondeado 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{92F79182-A741-45AA-B029-E7AB544C7506}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="25664160" y="3627120"/>
+          <a:ext cx="3025140" cy="891540"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T3. </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Homologación: Estandarizar descripciones para evitar inconsistencias (por ejemplo, diferencias de mayúsculas, espacios o abreviaturas).</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-CO" sz="1100" b="0">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>106680</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>3108960</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>22860</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="59" name="Rectángulo redondeado 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9B9AE1F5-EF2D-42E6-BB2B-E9C066EC3D95}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="25702260" y="4579620"/>
+          <a:ext cx="3002280" cy="929640"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T4. </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Generación de clave sustituta: Crear:</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>SK_CondicionPago</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>manteniendo idCondicionesDePago_T como clave natural.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:endParaRPr lang="es-CO" sz="1100" b="0">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>91440</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>137160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>3086100</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>91440</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="60" name="Rectángulo redondeado 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{06CAC060-851D-4CAB-A5F3-55A0F0365BEC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="25687020" y="5623560"/>
+          <a:ext cx="2994660" cy="685800"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T5</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>. Validación de integridad: Comprobar que todas las condiciones utilizadas posteriormente en la tabla de hechos existan en esta dimensión. </a:t>
+          </a:r>
+          <a:endParaRPr lang="es-CO" sz="1100" b="0">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </a:endParaRPr>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -1246,7 +2790,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagen 1"/>
+        <xdr:cNvPr id="2" name="Imagen 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -1534,26 +3084,28 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N36"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:P55"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="27.140625" customWidth="1"/>
-    <col min="4" max="4" width="53.85546875" customWidth="1"/>
-    <col min="6" max="6" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="45.28515625" customWidth="1"/>
-    <col min="10" max="10" width="27.140625" customWidth="1"/>
-    <col min="12" max="12" width="51.140625" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="4" max="4" width="53.88671875" customWidth="1"/>
+    <col min="6" max="6" width="29.109375" customWidth="1"/>
+    <col min="8" max="8" width="45.33203125" customWidth="1"/>
+    <col min="10" max="10" width="30.44140625" customWidth="1"/>
+    <col min="12" max="12" width="52.109375" customWidth="1"/>
+    <col min="14" max="14" width="41.5546875" customWidth="1"/>
+    <col min="16" max="16" width="45.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B2" s="9" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C2" s="9"/>
       <c r="D2" s="9"/>
@@ -1567,283 +3119,553 @@
       <c r="L2" s="9"/>
       <c r="M2" s="9"/>
       <c r="N2" s="9"/>
-    </row>
-    <row r="4" spans="1:14" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="O2" s="9"/>
+      <c r="P2" s="9"/>
+    </row>
+    <row r="4" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B4" s="10" t="s">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="C4" s="10"/>
       <c r="D4" s="10"/>
       <c r="F4" s="10" t="s">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="G4" s="10"/>
       <c r="H4" s="10"/>
       <c r="J4" s="10" t="s">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="K4" s="10"/>
       <c r="L4" s="10"/>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N4" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="O4" s="10"/>
+      <c r="P4" s="10"/>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+      <c r="N6" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B7" s="2" t="s">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D7" s="4"/>
       <c r="F7" s="2" t="s">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="H7" s="4"/>
       <c r="J7" s="2" t="s">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="L7" s="4"/>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N7" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="P7" s="4"/>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B8" s="1"/>
       <c r="D8" s="4"/>
       <c r="F8" s="1"/>
       <c r="H8" s="4"/>
       <c r="J8" s="1"/>
       <c r="L8" s="4"/>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N8" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="P8" s="4"/>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B9" s="3" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D9" s="4"/>
       <c r="F9" s="3" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H9" s="4"/>
       <c r="J9" s="3" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L9" s="4"/>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N9" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="P9" s="4"/>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B10" s="2" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="N10" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B11" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="F11" s="2"/>
+      <c r="J11" s="1"/>
+      <c r="N11" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B12" s="1"/>
       <c r="D12" s="5" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F12" s="1"/>
       <c r="H12" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="J12" s="1"/>
+        <v>5</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>2</v>
+      </c>
       <c r="L12" s="5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="N12" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="P12" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B13" s="3" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D13" s="4"/>
       <c r="F13" s="3" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H13" s="4"/>
-      <c r="J13" s="3" t="s">
-        <v>5</v>
+      <c r="J13" s="2" t="s">
+        <v>24</v>
       </c>
       <c r="L13" s="4"/>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N13" s="2"/>
+      <c r="P13" s="4"/>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B14" s="2" t="s">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="D14" s="4"/>
       <c r="F14" s="2" t="s">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="H14" s="4"/>
       <c r="J14" s="2" t="s">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="L14" s="4"/>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N14" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="P14" s="4"/>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B15" s="2" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="D15" s="4"/>
       <c r="F15" s="2" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="H15" s="4"/>
       <c r="J15" s="2" t="s">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="L15" s="4"/>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N15" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="P15" s="4"/>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="B16" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="D16" s="4"/>
+      <c r="F16" s="2" t="s">
+        <v>25</v>
+      </c>
       <c r="H16" s="4"/>
+      <c r="J16" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="L16" s="4"/>
-    </row>
-    <row r="17" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="N16" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="P16" s="4"/>
+    </row>
+    <row r="17" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B17" s="2" t="s">
+        <v>25</v>
+      </c>
       <c r="D17" s="4"/>
+      <c r="F17" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="H17" s="4"/>
+      <c r="J17" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="L17" s="4"/>
-    </row>
-    <row r="18" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="N17" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="P17" s="4"/>
+    </row>
+    <row r="18" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B18" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="D18" s="4"/>
+      <c r="F18" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="H18" s="4"/>
+      <c r="J18" s="2" t="s">
+        <v>13</v>
+      </c>
       <c r="L18" s="4"/>
-    </row>
-    <row r="19" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="N18" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="P18" s="4"/>
+    </row>
+    <row r="19" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B19" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="D19" s="4"/>
+      <c r="F19" s="2" t="s">
+        <v>13</v>
+      </c>
       <c r="H19" s="4"/>
+      <c r="J19" s="2" t="s">
+        <v>28</v>
+      </c>
       <c r="L19" s="4"/>
-    </row>
-    <row r="20" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="N19" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="P19" s="6"/>
+    </row>
+    <row r="20" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B20" s="2" t="s">
+        <v>28</v>
+      </c>
       <c r="D20" s="4"/>
+      <c r="F20" s="2" t="s">
+        <v>28</v>
+      </c>
       <c r="H20" s="4"/>
+      <c r="J20" s="2" t="s">
+        <v>29</v>
+      </c>
       <c r="L20" s="4"/>
-    </row>
-    <row r="21" spans="4:12" x14ac:dyDescent="0.25">
+      <c r="N20" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="P20" s="6"/>
+    </row>
+    <row r="21" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B21" s="2" t="s">
+        <v>29</v>
+      </c>
       <c r="D21" s="4"/>
+      <c r="F21" s="2" t="s">
+        <v>29</v>
+      </c>
       <c r="H21" s="4"/>
+      <c r="J21" s="2" t="s">
+        <v>30</v>
+      </c>
       <c r="L21" s="4"/>
-    </row>
-    <row r="26" spans="4:12" x14ac:dyDescent="0.25">
-      <c r="D26" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="H26" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="L26" s="5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="27" spans="4:12" x14ac:dyDescent="0.25">
-      <c r="D27" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H27" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L27" s="6" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="28" spans="4:12" x14ac:dyDescent="0.25">
-      <c r="D28" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="H28" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="L28" s="8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="29" spans="4:12" x14ac:dyDescent="0.25">
-      <c r="D29" s="6"/>
-      <c r="H29" s="6"/>
-      <c r="L29" s="6"/>
-    </row>
-    <row r="30" spans="4:12" x14ac:dyDescent="0.25">
-      <c r="D30" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="H30" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="L30" s="6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="31" spans="4:12" x14ac:dyDescent="0.25">
-      <c r="D31" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="H31" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="L31" s="8" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="32" spans="4:12" x14ac:dyDescent="0.25">
-      <c r="D32" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="H32" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="L32" s="8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="33" spans="4:12" x14ac:dyDescent="0.25">
-      <c r="D33" s="6"/>
-      <c r="H33" s="6"/>
-      <c r="L33" s="6"/>
-    </row>
-    <row r="34" spans="4:12" x14ac:dyDescent="0.25">
-      <c r="D34" s="6"/>
-      <c r="H34" s="6"/>
-      <c r="L34" s="6"/>
-    </row>
-    <row r="35" spans="4:12" x14ac:dyDescent="0.25">
-      <c r="D35" s="6"/>
-      <c r="H35" s="6"/>
-      <c r="L35" s="6"/>
-    </row>
-    <row r="36" spans="4:12" x14ac:dyDescent="0.25">
-      <c r="D36" s="7"/>
+      <c r="N21" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="P21" s="6"/>
+    </row>
+    <row r="22" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B22" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D22" s="4"/>
+      <c r="F22" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H22" s="4"/>
+      <c r="J22" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="L22" s="4"/>
+      <c r="N22" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="P22" s="6"/>
+    </row>
+    <row r="23" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B23" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D23" s="4"/>
+      <c r="F23" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H23" s="4"/>
+      <c r="L23" s="4"/>
+      <c r="N23" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="P23" s="6"/>
+    </row>
+    <row r="24" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="D24" s="4"/>
+      <c r="H24" s="4"/>
+      <c r="L24" s="4"/>
+      <c r="P24" s="6"/>
+    </row>
+    <row r="25" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="D25" s="4"/>
+      <c r="H25" s="4"/>
+      <c r="L25" s="4"/>
+      <c r="P25" s="6"/>
+    </row>
+    <row r="26" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="D26" s="4"/>
+      <c r="H26" s="4"/>
+      <c r="P26" s="6"/>
+    </row>
+    <row r="27" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="D27" s="4"/>
+      <c r="H27" s="4"/>
+      <c r="P27" s="6"/>
+    </row>
+    <row r="28" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="D28" s="4"/>
+      <c r="H28" s="4"/>
+      <c r="L28" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="P28" s="6"/>
+    </row>
+    <row r="29" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="D29" s="4"/>
+      <c r="H29" s="4"/>
+      <c r="L29" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="P29" s="6"/>
+    </row>
+    <row r="30" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="D30" s="4"/>
+      <c r="H30" s="4"/>
+      <c r="L30" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="P30" s="6"/>
+    </row>
+    <row r="31" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="H31" s="4"/>
+      <c r="L31" s="6"/>
+      <c r="P31" s="6"/>
+    </row>
+    <row r="32" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="H32" s="4"/>
+      <c r="L32" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="P32" s="6"/>
+    </row>
+    <row r="33" spans="4:16" x14ac:dyDescent="0.3">
+      <c r="H33" s="4"/>
+      <c r="L33" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="P33" s="6"/>
+    </row>
+    <row r="34" spans="4:16" x14ac:dyDescent="0.3">
+      <c r="H34" s="4"/>
+      <c r="L34" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="P34" s="6"/>
+    </row>
+    <row r="35" spans="4:16" x14ac:dyDescent="0.3">
+      <c r="D35" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H35" s="4"/>
+      <c r="P35" s="6"/>
+    </row>
+    <row r="36" spans="4:16" x14ac:dyDescent="0.3">
+      <c r="D36" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="H36" s="4"/>
+      <c r="P36" s="12"/>
+    </row>
+    <row r="37" spans="4:16" x14ac:dyDescent="0.3">
+      <c r="D37" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H37" s="4"/>
+      <c r="P37" s="12"/>
+    </row>
+    <row r="38" spans="4:16" x14ac:dyDescent="0.3">
+      <c r="D38" s="6"/>
+      <c r="H38" s="4"/>
+      <c r="P38" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="39" spans="4:16" x14ac:dyDescent="0.3">
+      <c r="D39" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="H39" s="4"/>
+      <c r="P39" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="40" spans="4:16" x14ac:dyDescent="0.3">
+      <c r="D40" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="H40" s="4"/>
+      <c r="P40" s="8" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="41" spans="4:16" x14ac:dyDescent="0.3">
+      <c r="D41" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H41" s="4"/>
+      <c r="P41" s="6"/>
+    </row>
+    <row r="42" spans="4:16" x14ac:dyDescent="0.3">
+      <c r="D42" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="P42" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="43" spans="4:16" x14ac:dyDescent="0.3">
+      <c r="D43" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="P43" s="11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="44" spans="4:16" x14ac:dyDescent="0.3">
+      <c r="D44" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="P44" s="8" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="45" spans="4:16" x14ac:dyDescent="0.3">
+      <c r="D45" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="P45" s="11" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="46" spans="4:16" x14ac:dyDescent="0.3">
+      <c r="D46" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="H46" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="47" spans="4:16" x14ac:dyDescent="0.3">
+      <c r="H47" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="48" spans="4:16" x14ac:dyDescent="0.3">
+      <c r="H48" s="8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="49" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H49" s="6"/>
+    </row>
+    <row r="50" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H50" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="51" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H51" s="11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="52" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H52" s="8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="53" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H53" s="6"/>
+    </row>
+    <row r="54" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H54" s="6"/>
+    </row>
+    <row r="55" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H55" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="B2:N2"/>
+  <mergeCells count="5">
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="F4:H4"/>
     <mergeCell ref="J4:L4"/>
+    <mergeCell ref="N4:P4"/>
+    <mergeCell ref="B2:P2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
@@ -1852,9 +3674,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
diseno etl dimensiones faltantes
</commit_message>
<xml_diff>
--- a/Segundo entregable/PlantillaDisenioETL.xlsx
+++ b/Segundo entregable/PlantillaDisenioETL.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Documents\GitHub\entrega_proyecto_MIAD_modelado_datos\Segundo entregable\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fabrizio.cucina\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BA3F12E-9188-4992-AA38-49C18921EADF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2B29A92-6E2A-4A43-AFE0-13C1E8EBAA8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,44 +16,28 @@
     <sheet name="PlantillaDiseñoETL" sheetId="1" r:id="rId1"/>
     <sheet name="Ejemplo" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="52">
-  <si>
-    <t>Campos a incluir:</t>
-  </si>
-  <si>
-    <t>*…</t>
-  </si>
-  <si>
-    <t>Campos No incluidos:</t>
-  </si>
-  <si>
-    <t>Fuente de datos:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Extraer información de </t>
-  </si>
-  <si>
-    <t>2. Transformaciones</t>
-  </si>
-  <si>
-    <t>3. Carga de los datos</t>
-  </si>
-  <si>
-    <t>Destino de los datos:</t>
-  </si>
-  <si>
-    <t>Campos a cargar:</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="95">
   <si>
     <t>Inspirada en el trabajo realizado por el Grupo Krusty_Brand202214</t>
   </si>
@@ -77,18 +61,129 @@
     <t>DimFecha</t>
   </si>
   <si>
+    <t>DimProveedor</t>
+  </si>
+  <si>
+    <t>DimPlan</t>
+  </si>
+  <si>
+    <t>DimCondicionPago</t>
+  </si>
+  <si>
+    <t>Fuente de datos:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Extraer información de </t>
+  </si>
+  <si>
     <t>* FuentePlanesBeneficio_Copia_E</t>
   </si>
   <si>
+    <t>* FuenteCondicionesPago_Copia_E</t>
+  </si>
+  <si>
+    <t>* FuenteTiposBeneficio_Copia_E</t>
+  </si>
+  <si>
+    <t>Campos a incluir:</t>
+  </si>
+  <si>
     <t>* Fecha</t>
   </si>
   <si>
+    <t>* idProveedor_T</t>
+  </si>
+  <si>
+    <t>* idPlan_T</t>
+  </si>
+  <si>
+    <t>* idCondicionesDePago_T</t>
+  </si>
+  <si>
+    <t>*…</t>
+  </si>
+  <si>
+    <t>* Tipo</t>
+  </si>
+  <si>
+    <t>2. Transformaciones</t>
+  </si>
+  <si>
+    <t>Campos No incluidos:</t>
+  </si>
+  <si>
+    <t>* Descripcion</t>
+  </si>
+  <si>
+    <t>* idTipoBeneficio_T</t>
+  </si>
+  <si>
+    <t>* idAreaDeServicio_T</t>
+  </si>
+  <si>
+    <t>* idCondicionesDePagoCopago_T</t>
+  </si>
+  <si>
+    <t>* idCondicionesDePagoCoseguro_T</t>
+  </si>
+  <si>
+    <t>* Nombre</t>
+  </si>
+  <si>
+    <t>* UnidadDelLimite</t>
+  </si>
+  <si>
+    <t>* EsEHB</t>
+  </si>
+  <si>
+    <t>* idNivelServicio_T</t>
+  </si>
+  <si>
+    <t>* EstaCubiertoPorSeguro</t>
+  </si>
+  <si>
+    <t>* valorCopago</t>
+  </si>
+  <si>
+    <t>* TieneLimiteCuantitativo</t>
+  </si>
+  <si>
+    <t>* valorCoseguro</t>
+  </si>
+  <si>
+    <t>* ExcluidoDelDesembolsoMaximoDentroDeLaRed</t>
+  </si>
+  <si>
+    <t>* cantidadLimite</t>
+  </si>
+  <si>
+    <t>* ExcluidoDelDesembolsoMaximoFueraDeLaRed</t>
+  </si>
+  <si>
+    <t>3. Carga de los datos</t>
+  </si>
+  <si>
+    <t>Destino de los datos:</t>
+  </si>
+  <si>
+    <t>* DimPlan</t>
+  </si>
+  <si>
+    <t>Campos a cargar:</t>
+  </si>
+  <si>
+    <t>* SK_Plan</t>
+  </si>
+  <si>
     <t>* DimFecha</t>
   </si>
   <si>
     <t>* SK_Fecha</t>
   </si>
   <si>
+    <t>* DimCondicionPago</t>
+  </si>
+  <si>
     <t>* Año</t>
   </si>
   <si>
@@ -104,39 +199,6 @@
     <t>* Día</t>
   </si>
   <si>
-    <t>DimProveedor</t>
-  </si>
-  <si>
-    <t>* idProveedor_T</t>
-  </si>
-  <si>
-    <t>* idPlan_T</t>
-  </si>
-  <si>
-    <t>* idTipoBeneficio_T</t>
-  </si>
-  <si>
-    <t>* idAreaDeServicio_T</t>
-  </si>
-  <si>
-    <t>* idCondicionesDePagoCopago_T</t>
-  </si>
-  <si>
-    <t>* idCondicionesDePagoCoseguro_T</t>
-  </si>
-  <si>
-    <t>* idNivelServicio_T</t>
-  </si>
-  <si>
-    <t>* valorCopago</t>
-  </si>
-  <si>
-    <t>* valorCoseguro</t>
-  </si>
-  <si>
-    <t>* cantidadLimite</t>
-  </si>
-  <si>
     <t>* DimProveedor</t>
   </si>
   <si>
@@ -146,55 +208,133 @@
     <t xml:space="preserve">* idProveedor_T </t>
   </si>
   <si>
-    <t>DimPlan</t>
-  </si>
-  <si>
-    <t>* DimPlan</t>
-  </si>
-  <si>
-    <t>* SK_Plan</t>
-  </si>
-  <si>
-    <t>DimCondicionPago</t>
-  </si>
-  <si>
-    <t>* FuenteTiposBeneficio_Copia_E</t>
-  </si>
-  <si>
-    <t>* idCondicionesDePago_T</t>
-  </si>
-  <si>
-    <t>* FuenteCondicionesPago_Copia_E</t>
-  </si>
-  <si>
-    <t>* Descripcion</t>
-  </si>
-  <si>
-    <t>* Nombre</t>
-  </si>
-  <si>
-    <t>* UnidadDelLimite</t>
-  </si>
-  <si>
-    <t>* EsEHB</t>
-  </si>
-  <si>
-    <t>* EstaCubiertoPorSeguro</t>
-  </si>
-  <si>
-    <t>* TieneLimiteCuantitativo</t>
-  </si>
-  <si>
-    <t>* ExcluidoDelDesembolsoMaximoDentroDeLaRed</t>
-  </si>
-  <si>
-    <t>* ExcluidoDelDesembolsoMaximoFueraDeLaRed</t>
-  </si>
-  <si>
-    <t>* DimCondicionPago</t>
-  </si>
-  <si>
-    <t>* Tipo</t>
+    <t>DimAreaServicio  (historia Tipo 2)</t>
+  </si>
+  <si>
+    <t>* FuenteAreasDeServicio_Copia_E</t>
+  </si>
+  <si>
+    <t>idAreaServicio_T, NombreAreaDeServicio, idGeografía_T, Estado, Condado, PoblacionAct, Area, Densidad, Fecha</t>
+  </si>
+  <si>
+    <t>Ninguno</t>
+  </si>
+  <si>
+    <t>DimAreaServicio</t>
+  </si>
+  <si>
+    <t>idAreaServicio_T</t>
+  </si>
+  <si>
+    <t>NombreAreaDeServicio</t>
+  </si>
+  <si>
+    <t>idGeografía_T</t>
+  </si>
+  <si>
+    <t>Estado</t>
+  </si>
+  <si>
+    <t>Condado</t>
+  </si>
+  <si>
+    <t>PoblacionAct</t>
+  </si>
+  <si>
+    <t>Area</t>
+  </si>
+  <si>
+    <t>Densidad</t>
+  </si>
+  <si>
+    <t>ValidoDesde</t>
+  </si>
+  <si>
+    <t>ValidoHasta</t>
+  </si>
+  <si>
+    <t>Actual</t>
+  </si>
+  <si>
+    <t>SK_AreaServicio</t>
+  </si>
+  <si>
+    <t>DimTipoBeneficio  (historia Tipo 2)</t>
+  </si>
+  <si>
+    <t>idTipoBeneficio_T, Nombre, UnidadDelLimite, EsEHB, EstaCubiertoPorSeguro, TieneLimiteCuantitativo, ExcluidoDelDesembolsoMaximoDentroDeLaRed, ExcluidoDelDesembolsoMaximoFueraDeLaRed, Fecha</t>
+  </si>
+  <si>
+    <t>Ninguno.</t>
+  </si>
+  <si>
+    <t>DimTipoBeneficio</t>
+  </si>
+  <si>
+    <t>SK_TipoBeneficio</t>
+  </si>
+  <si>
+    <t>idTipoBeneficio_T</t>
+  </si>
+  <si>
+    <t>Nombre</t>
+  </si>
+  <si>
+    <t>UnidadDelLimite</t>
+  </si>
+  <si>
+    <t>EsEHB</t>
+  </si>
+  <si>
+    <t>EstaCubiertoPorSeguro</t>
+  </si>
+  <si>
+    <t>TieneLimiteCuantitativo</t>
+  </si>
+  <si>
+    <t>ExcluidoDelDesembolsoMaximoDentroDeLaRed</t>
+  </si>
+  <si>
+    <t>ExcluidoDelDesembolsoMaximoFueraDeLaRed</t>
+  </si>
+  <si>
+    <t>Hecho_OfertaPlanBeneficio</t>
+  </si>
+  <si>
+    <t>* FuentePlanesBeneficio_Copia_E (+ dimensiones ya cargadas para los lookups)</t>
+  </si>
+  <si>
+    <t>SK_Fecha</t>
+  </si>
+  <si>
+    <t>SK_Plan</t>
+  </si>
+  <si>
+    <t>SK_Proveedor</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> SK_AreaServicio</t>
+  </si>
+  <si>
+    <t>SK_CondicionPagoCopago</t>
+  </si>
+  <si>
+    <t>SK_CondicionPagoCoseguro</t>
+  </si>
+  <si>
+    <t>idNivelServicio_T</t>
+  </si>
+  <si>
+    <t>valorCopago</t>
+  </si>
+  <si>
+    <t>valorCoseguro</t>
+  </si>
+  <si>
+    <t>cantidadLimite</t>
+  </si>
+  <si>
+    <t>ConteoOfertaBeneficio</t>
   </si>
 </sst>
 </file>
@@ -286,7 +426,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -298,16 +438,23 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2765,6 +2912,2173 @@
               <a:srgbClr val="FF0000"/>
             </a:solidFill>
           </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1821180</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1824990</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="3" name="Conector recto de flecha 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{213930EE-D81A-4083-85F6-B680ACBEA2A2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="5334000" y="5448300"/>
+          <a:ext cx="3810" cy="754380"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1562100</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1565910</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>137160</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="6" name="Conector recto de flecha 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{27B7B666-DCF5-4388-8837-9579E14527C4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="12367260" y="7330440"/>
+          <a:ext cx="3810" cy="853440"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1790700</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1798321</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="11" name="Conector recto de flecha 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9B1B6306-7838-462D-9587-676267CCB497}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="19362420" y="4522470"/>
+          <a:ext cx="7621" cy="445770"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>1722120</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>1722121</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="14" name="Conector recto de flecha 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{04B09DE3-CAD0-4BFE-A523-33D8F751028F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="27287220" y="6362700"/>
+          <a:ext cx="1" cy="392430"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>472441</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>2887981</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="15" name="Rectángulo redondeado 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5FA5BC2B-0850-41CB-AA6A-AD43B820EC73}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4015741" y="1249680"/>
+          <a:ext cx="2415540" cy="308610"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="CCCCFF"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>* FuenteAreasDeServicio_Copia_E </a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>15240</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>121920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>472441</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="19" name="Conector recto de flecha 18">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{858B73DD-5140-4F2E-AF97-F2E6F4D822FF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="15" idx="1"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1" flipV="1">
+          <a:off x="2773680" y="1402080"/>
+          <a:ext cx="1242061" cy="1905"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>167641</xdr:colOff>
+      <xdr:row>60</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>3444241</xdr:colOff>
+      <xdr:row>62</xdr:row>
+      <xdr:rowOff>160020</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="21" name="Rectángulo redondeado 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3F1C33F7-BEA5-49D7-979B-2FABD205DD8D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3710941" y="11003280"/>
+          <a:ext cx="3276600" cy="495300"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T1. Eliminar filas totalmente duplicadas (el área se repite muchas veces en la fuente).</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>220980</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>129540</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>3390900</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>106680</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="24" name="Rectángulo redondeado 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9C635D0E-315A-4174-9BCB-3DD35514DCF7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3764280" y="12199620"/>
+          <a:ext cx="3169920" cy="525780"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T3. Estandarizar Estado y Condado (mayúsculas/espacios).</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1676401</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1680211</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="25" name="Conector recto de flecha 24">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{02A868DC-1CEA-48FD-AB33-BDB13067A7EC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="15" idx="2"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="5219701" y="1558290"/>
+          <a:ext cx="3810" cy="491490"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>198121</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>80010</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>3368041</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="27" name="Rectángulo redondeado 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{09117096-2EA5-4600-8CF9-E01A6D84C117}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3741421" y="11601450"/>
+          <a:ext cx="3169920" cy="476250"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T2. Corregir valores inválidos: Area negativa y PoblacionAct/Densidad atípicas.</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>68580</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>3573780</xdr:colOff>
+      <xdr:row>73</xdr:row>
+      <xdr:rowOff>106680</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="30" name="Rectángulo redondeado 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D80FD955-63AF-4C54-ABA4-B9C3F2DC4C14}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3611880" y="12786360"/>
+          <a:ext cx="3505200" cy="670560"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T4. Historia Tipo 2: agregar ValidoDesde, ValidoHasta (2199-12-31) y Actual; cerrar/insertar versión cuando cambien atributos (p. ej. PoblacionAct/Densidad).</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>516255</xdr:colOff>
+      <xdr:row>73</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>3131820</xdr:colOff>
+      <xdr:row>75</xdr:row>
+      <xdr:rowOff>110490</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="31" name="Rectángulo redondeado 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A81AC4B1-13A5-473E-ADEF-699B744D2B0C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4059555" y="13517880"/>
+          <a:ext cx="2615565" cy="308610"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T5. Generar SK_AreaServicio (una por versión).</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1821180</xdr:colOff>
+      <xdr:row>77</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1824990</xdr:colOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="32" name="Conector recto de flecha 31">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{56CA266C-4D66-44C5-BFCE-D47D9E8540F6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="5364480" y="5448300"/>
+          <a:ext cx="3810" cy="754380"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>472441</xdr:colOff>
+      <xdr:row>61</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>2887981</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="34" name="Rectángulo redondeado 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B45F1B63-5A98-4C2E-B474-62C3D3479487}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4015741" y="10027920"/>
+          <a:ext cx="2415540" cy="308610"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="CCCCFF"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" b="0" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>* FuenteTiposBeneficio_Copia_E</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>15240</xdr:colOff>
+      <xdr:row>62</xdr:row>
+      <xdr:rowOff>121920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>472441</xdr:colOff>
+      <xdr:row>62</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="35" name="Conector recto de flecha 34">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6985F0C4-C7AC-47D6-8E10-C726A4671E83}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="34" idx="1"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1" flipV="1">
+          <a:off x="2773680" y="10180320"/>
+          <a:ext cx="1242061" cy="1905"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>167641</xdr:colOff>
+      <xdr:row>67</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>71</xdr:row>
+      <xdr:rowOff>83820</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="36" name="Rectángulo redondeado 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{68B3421C-D433-477F-8EE2-CC122F9B20B4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10972801" y="12283440"/>
+          <a:ext cx="2941320" cy="784860"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T1. Estandarizar banderas a un dominio único (Sí/No): Yes/Si-&gt;Sí, No/Nein-&gt;No, True-&gt;Sí, False-&gt;No; depurar valores atípicos ('Algunas veces').</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>182880</xdr:colOff>
+      <xdr:row>74</xdr:row>
+      <xdr:rowOff>175260</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>3070860</xdr:colOff>
+      <xdr:row>76</xdr:row>
+      <xdr:rowOff>121920</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="38" name="Rectángulo redondeado 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B638798D-22AB-4D53-8FEC-39F816010855}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10988040" y="13708380"/>
+          <a:ext cx="2887980" cy="312420"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T3. Eliminar duplicados de idTipoBeneficio_T.</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1676401</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1680211</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="39" name="Conector recto de flecha 38">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D0159292-CE6D-4652-980D-FFD04F743998}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="34" idx="2"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="5219701" y="10336530"/>
+          <a:ext cx="3810" cy="491490"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>175261</xdr:colOff>
+      <xdr:row>71</xdr:row>
+      <xdr:rowOff>110490</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>3086101</xdr:colOff>
+      <xdr:row>74</xdr:row>
+      <xdr:rowOff>91440</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="43" name="Rectángulo redondeado 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{61A912BA-9651-406C-8C8F-44D127368EB9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10980421" y="13094970"/>
+          <a:ext cx="2910840" cy="529590"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T2. Limpiar UnidadDelLimite: quitar vacíos y corregir cadenas corruptas/triplicadas.</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>45720</xdr:colOff>
+      <xdr:row>77</xdr:row>
+      <xdr:rowOff>68580</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>3086100</xdr:colOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="44" name="Rectángulo redondeado 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{14187333-2172-43D5-B605-A7CE3F0F3110}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10850880" y="14150340"/>
+          <a:ext cx="3040380" cy="807720"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T4. Historia Tipo 2: ValidoDesde, ValidoHasta (2199-12-31) y Actual; cerrar/insertar versión cuando cambien cobertura, límites o exclusiones.</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>249555</xdr:colOff>
+      <xdr:row>82</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>2842260</xdr:colOff>
+      <xdr:row>84</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="45" name="Rectángulo redondeado 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E498831B-E4A0-4858-A202-A9689DE544FE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11054715" y="15057120"/>
+          <a:ext cx="2592705" cy="438150"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T5. Generar SK_TipoBeneficio (una por versión).</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1821180</xdr:colOff>
+      <xdr:row>84</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1824990</xdr:colOff>
+      <xdr:row>88</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="46" name="Conector recto de flecha 45">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{22283289-8822-4EFA-950B-6C282D5B5F22}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="5364480" y="14226540"/>
+          <a:ext cx="3810" cy="754380"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>716280</xdr:colOff>
+      <xdr:row>60</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>198119</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="47" name="Rectángulo redondeado 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8536CBAD-7BFC-4903-A5A4-31D11EC4E915}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="21861780" y="11018520"/>
+          <a:ext cx="3116579" cy="579120"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="CCCCFF"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" b="0" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>* FuentePlanesBeneficio_Copia_E (+ dimensiones ya cargadas para los lookups)</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-GB">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+            <a:effectLst/>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>45720</xdr:colOff>
+      <xdr:row>61</xdr:row>
+      <xdr:rowOff>137160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>716280</xdr:colOff>
+      <xdr:row>61</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="61" name="Conector recto de flecha 60">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{25428300-B7D2-4EFA-8C11-435D42437ECC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="47" idx="1"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1" flipV="1">
+          <a:off x="21191220" y="11292840"/>
+          <a:ext cx="670560" cy="15240"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>167641</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>68</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="62" name="Rectángulo redondeado 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6A8619D7-6B06-439E-930D-F06CBF3B2572}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="22098001" y="12100560"/>
+          <a:ext cx="2682240" cy="365760"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T1. Eliminar filas totalmente duplicadas.</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>182880</xdr:colOff>
+      <xdr:row>73</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>76</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="63" name="Rectángulo redondeado 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5858A45F-0363-4254-869D-38DF5FB92399}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="22113240" y="13395960"/>
+          <a:ext cx="2667000" cy="541020"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T3. Derivar SK_Fecha desde la Fecha estandarizada (cruce con DimFecha).</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>1485900</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>1489710</xdr:colOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="64" name="Conector recto de flecha 63">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5B52704D-20B6-4088-B44E-A16B75942718}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="47" idx="2"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="23416260" y="11597640"/>
+          <a:ext cx="3810" cy="297180"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>129541</xdr:colOff>
+      <xdr:row>68</xdr:row>
+      <xdr:rowOff>129540</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>2804161</xdr:colOff>
+      <xdr:row>73</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="65" name="Rectángulo redondeado 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8737B5F5-15D8-418B-9600-97D11856AB4C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="22059901" y="12565380"/>
+          <a:ext cx="2674620" cy="845820"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T2. Validar valorCopago/valorCoseguro contra el rango del negocio (marcar outliers, p. ej. copago 3500 &gt; 3300 en 2018).</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>76</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>2842260</xdr:colOff>
+      <xdr:row>80</xdr:row>
+      <xdr:rowOff>137160</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="66" name="Rectángulo redondeado 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{16F6172F-4BC4-4D22-AF82-27E7A9C9D759}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="21968460" y="13959840"/>
+          <a:ext cx="2804160" cy="807720"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T4. Lookup por llave de negocio (_T) para traer las SK: Plan, Proveedor y CondicionPago (rol copago y rol coseguro).</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>81915</xdr:colOff>
+      <xdr:row>93</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>2674620</xdr:colOff>
+      <xdr:row>96</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="67" name="Rectángulo redondeado 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{97899DDE-5215-43A8-B354-526244180F2D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="22012275" y="17068800"/>
+          <a:ext cx="2592705" cy="533400"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T7. Asignar comodín SK = 0 a las FK sin coincidencia (integridad referencial).</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>1337310</xdr:colOff>
+      <xdr:row>99</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>1341120</xdr:colOff>
+      <xdr:row>102</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="68" name="Conector recto de flecha 67">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4C1D1A5B-9DDB-499C-9FE1-5D812D736E73}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="23267670" y="18272760"/>
+          <a:ext cx="3810" cy="411480"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>97155</xdr:colOff>
+      <xdr:row>86</xdr:row>
+      <xdr:rowOff>53340</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>2689860</xdr:colOff>
+      <xdr:row>89</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="79" name="Rectángulo redondeado 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7F9F1ED5-4A4D-4A3E-8115-0CDFE0C90BE9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="22027515" y="15781020"/>
+          <a:ext cx="2592705" cy="525780"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T6. idNivelServicio_T se conserva como dimensión degenerada (sin lookup).</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>89535</xdr:colOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>2682240</xdr:colOff>
+      <xdr:row>85</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="80" name="Rectángulo redondeado 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{91E5468E-FFCB-47FE-B4CD-18C72AA3BFDA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="22019895" y="14859000"/>
+          <a:ext cx="2592705" cy="853440"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T5. Lookup Tipo 2 para AreaServicio y TipoBeneficio: tomar la versión vigente en la Fecha de la oferta (Fecha entre ValidoDesde y ValidoHasta).</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
+      <xdr:row>89</xdr:row>
+      <xdr:rowOff>121920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>2659380</xdr:colOff>
+      <xdr:row>92</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="81" name="Rectángulo redondeado 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{07B35E63-D317-4309-AE81-E47F3A0611C8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="21997035" y="16398240"/>
+          <a:ext cx="2592705" cy="487680"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T6. idNivelServicio_T se conserva como dimensión degenerada (sin lookup).</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>59055</xdr:colOff>
+      <xdr:row>96</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>2651760</xdr:colOff>
+      <xdr:row>99</xdr:row>
+      <xdr:rowOff>129540</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="82" name="Rectángulo redondeado 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1EAAEF5A-82C1-4473-9C3C-17849CFCE0A2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="21989415" y="17701260"/>
+          <a:ext cx="2592705" cy="533400"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T8. Calcular ConteoOfertaBeneficio = 1 por fila (para conteos distintos).</a:t>
+          </a:r>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -3085,106 +5399,106 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P55"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:P119"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="2" max="2" width="28.77734375" customWidth="1"/>
     <col min="4" max="4" width="53.88671875" customWidth="1"/>
     <col min="6" max="6" width="29.109375" customWidth="1"/>
     <col min="8" max="8" width="45.33203125" customWidth="1"/>
     <col min="10" max="10" width="30.44140625" customWidth="1"/>
     <col min="12" max="12" width="52.109375" customWidth="1"/>
     <col min="14" max="14" width="41.5546875" customWidth="1"/>
-    <col min="16" max="16" width="45.77734375" customWidth="1"/>
+    <col min="16" max="16" width="45.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="B2" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
-      <c r="I2" s="9"/>
-      <c r="J2" s="9"/>
-      <c r="K2" s="9"/>
-      <c r="L2" s="9"/>
-      <c r="M2" s="9"/>
-      <c r="N2" s="9"/>
-      <c r="O2" s="9"/>
-      <c r="P2" s="9"/>
+      <c r="B2" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="11"/>
+      <c r="J2" s="11"/>
+      <c r="K2" s="11"/>
+      <c r="L2" s="11"/>
+      <c r="M2" s="11"/>
+      <c r="N2" s="11"/>
+      <c r="O2" s="11"/>
+      <c r="P2" s="11"/>
     </row>
     <row r="4" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B4" s="10" t="s">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="C4" s="10"/>
       <c r="D4" s="10"/>
       <c r="F4" s="10" t="s">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="G4" s="10"/>
       <c r="H4" s="10"/>
       <c r="J4" s="10" t="s">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="K4" s="10"/>
       <c r="L4" s="10"/>
       <c r="N4" s="10" t="s">
-        <v>38</v>
+        <v>5</v>
       </c>
       <c r="O4" s="10"/>
       <c r="P4" s="10"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B7" s="2" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D7" s="4"/>
       <c r="F7" s="2" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H7" s="4"/>
       <c r="J7" s="2" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="L7" s="4"/>
       <c r="N7" s="2" t="s">
-        <v>41</v>
+        <v>9</v>
       </c>
       <c r="P7" s="4"/>
     </row>
@@ -3196,85 +5510,85 @@
       <c r="J8" s="1"/>
       <c r="L8" s="4"/>
       <c r="N8" s="2" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="P8" s="4"/>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B9" s="3" t="s">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="D9" s="4"/>
       <c r="F9" s="3" t="s">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="H9" s="4"/>
       <c r="J9" s="3" t="s">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="L9" s="4"/>
       <c r="N9" s="3" t="s">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="P9" s="4"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>22</v>
-      </c>
       <c r="J10" s="2" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>40</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B11" s="2" t="s">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="F11" s="2"/>
       <c r="J11" s="1"/>
       <c r="N11" s="2" t="s">
-        <v>51</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B12" s="1"/>
       <c r="D12" s="5" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="F12" s="1"/>
       <c r="H12" s="5" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="L12" s="5" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="P12" s="5" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B13" s="3" t="s">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="D13" s="4"/>
       <c r="F13" s="3" t="s">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="H13" s="4"/>
       <c r="J13" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="L13" s="4"/>
       <c r="N13" s="2"/>
@@ -3282,101 +5596,101 @@
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B14" s="2" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D14" s="4"/>
       <c r="F14" s="2" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="H14" s="4"/>
       <c r="J14" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="L14" s="4"/>
       <c r="N14" s="3" t="s">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="P14" s="4"/>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B15" s="2" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="D15" s="4"/>
       <c r="F15" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H15" s="4"/>
       <c r="J15" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="L15" s="4"/>
       <c r="N15" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="P15" s="4"/>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B16" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D16" s="4"/>
       <c r="F16" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="H16" s="4"/>
       <c r="J16" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="L16" s="4"/>
       <c r="N16" s="2" t="s">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="P16" s="4"/>
     </row>
     <row r="17" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B17" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D17" s="4"/>
       <c r="F17" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="H17" s="4"/>
       <c r="J17" s="2" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="L17" s="4"/>
       <c r="N17" s="2" t="s">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="P17" s="4"/>
     </row>
     <row r="18" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B18" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D18" s="4"/>
       <c r="F18" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="H18" s="4"/>
       <c r="J18" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="L18" s="4"/>
       <c r="N18" s="2" t="s">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="P18" s="4"/>
     </row>
     <row r="19" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B19" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D19" s="4"/>
       <c r="F19" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H19" s="4"/>
       <c r="J19" s="2" t="s">
@@ -3384,7 +5698,7 @@
       </c>
       <c r="L19" s="4"/>
       <c r="N19" s="2" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="P19" s="6"/>
     </row>
@@ -3398,62 +5712,62 @@
       </c>
       <c r="H20" s="4"/>
       <c r="J20" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L20" s="4"/>
       <c r="N20" s="2" t="s">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="P20" s="6"/>
     </row>
     <row r="21" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B21" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D21" s="4"/>
       <c r="F21" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H21" s="4"/>
       <c r="J21" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="L21" s="4"/>
       <c r="N21" s="2" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="P21" s="6"/>
     </row>
     <row r="22" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B22" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D22" s="4"/>
       <c r="F22" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H22" s="4"/>
       <c r="J22" s="2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="L22" s="4"/>
       <c r="N22" s="2" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="P22" s="6"/>
     </row>
     <row r="23" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B23" s="2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D23" s="4"/>
       <c r="F23" s="2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="H23" s="4"/>
       <c r="L23" s="4"/>
       <c r="N23" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="P23" s="6"/>
     </row>
@@ -3483,7 +5797,7 @@
       <c r="D28" s="4"/>
       <c r="H28" s="4"/>
       <c r="L28" s="5" t="s">
-        <v>6</v>
+        <v>36</v>
       </c>
       <c r="P28" s="6"/>
     </row>
@@ -3491,7 +5805,7 @@
       <c r="D29" s="4"/>
       <c r="H29" s="4"/>
       <c r="L29" s="6" t="s">
-        <v>7</v>
+        <v>37</v>
       </c>
       <c r="P29" s="6"/>
     </row>
@@ -3499,7 +5813,7 @@
       <c r="D30" s="4"/>
       <c r="H30" s="4"/>
       <c r="L30" s="8" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="P30" s="6"/>
     </row>
@@ -3511,156 +5825,644 @@
     <row r="32" spans="2:16" x14ac:dyDescent="0.3">
       <c r="H32" s="4"/>
       <c r="L32" s="6" t="s">
-        <v>8</v>
+        <v>39</v>
       </c>
       <c r="P32" s="6"/>
     </row>
     <row r="33" spans="4:16" x14ac:dyDescent="0.3">
       <c r="H33" s="4"/>
-      <c r="L33" s="11" t="s">
-        <v>37</v>
+      <c r="L33" s="9" t="s">
+        <v>40</v>
       </c>
       <c r="P33" s="6"/>
     </row>
     <row r="34" spans="4:16" x14ac:dyDescent="0.3">
       <c r="H34" s="4"/>
       <c r="L34" s="8" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="P34" s="6"/>
     </row>
     <row r="35" spans="4:16" x14ac:dyDescent="0.3">
       <c r="D35" s="5" t="s">
-        <v>6</v>
+        <v>36</v>
       </c>
       <c r="H35" s="4"/>
       <c r="P35" s="6"/>
     </row>
     <row r="36" spans="4:16" x14ac:dyDescent="0.3">
       <c r="D36" s="6" t="s">
-        <v>7</v>
+        <v>37</v>
       </c>
       <c r="H36" s="4"/>
-      <c r="P36" s="12"/>
+      <c r="P36" s="7"/>
     </row>
     <row r="37" spans="4:16" x14ac:dyDescent="0.3">
       <c r="D37" s="8" t="s">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="H37" s="4"/>
-      <c r="P37" s="12"/>
+      <c r="P37" s="7"/>
     </row>
     <row r="38" spans="4:16" x14ac:dyDescent="0.3">
       <c r="D38" s="6"/>
       <c r="H38" s="4"/>
       <c r="P38" s="5" t="s">
-        <v>6</v>
+        <v>36</v>
       </c>
     </row>
     <row r="39" spans="4:16" x14ac:dyDescent="0.3">
       <c r="D39" s="6" t="s">
-        <v>8</v>
+        <v>39</v>
       </c>
       <c r="H39" s="4"/>
       <c r="P39" s="6" t="s">
-        <v>7</v>
+        <v>37</v>
       </c>
     </row>
     <row r="40" spans="4:16" x14ac:dyDescent="0.3">
       <c r="D40" s="8" t="s">
-        <v>15</v>
+        <v>42</v>
       </c>
       <c r="H40" s="4"/>
       <c r="P40" s="8" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
     </row>
     <row r="41" spans="4:16" x14ac:dyDescent="0.3">
       <c r="D41" s="8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H41" s="4"/>
       <c r="P41" s="6"/>
     </row>
     <row r="42" spans="4:16" x14ac:dyDescent="0.3">
       <c r="D42" s="8" t="s">
-        <v>16</v>
+        <v>44</v>
       </c>
       <c r="P42" s="6" t="s">
-        <v>8</v>
+        <v>39</v>
       </c>
     </row>
     <row r="43" spans="4:16" x14ac:dyDescent="0.3">
       <c r="D43" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="P43" s="11" t="s">
-        <v>40</v>
+        <v>45</v>
+      </c>
+      <c r="P43" s="9" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="44" spans="4:16" x14ac:dyDescent="0.3">
       <c r="D44" s="8" t="s">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="P44" s="8" t="s">
-        <v>51</v>
+        <v>17</v>
       </c>
     </row>
     <row r="45" spans="4:16" x14ac:dyDescent="0.3">
       <c r="D45" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="P45" s="11" t="s">
-        <v>42</v>
+        <v>47</v>
+      </c>
+      <c r="P45" s="9" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="46" spans="4:16" x14ac:dyDescent="0.3">
       <c r="D46" s="8" t="s">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="H46" s="5" t="s">
-        <v>6</v>
+        <v>36</v>
       </c>
     </row>
     <row r="47" spans="4:16" x14ac:dyDescent="0.3">
       <c r="H47" s="6" t="s">
-        <v>7</v>
+        <v>37</v>
       </c>
     </row>
     <row r="48" spans="4:16" x14ac:dyDescent="0.3">
       <c r="H48" s="8" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="49" spans="8:8" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="49" spans="2:14" x14ac:dyDescent="0.3">
       <c r="H49" s="6"/>
     </row>
-    <row r="50" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:14" x14ac:dyDescent="0.3">
       <c r="H50" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="51" spans="8:8" x14ac:dyDescent="0.3">
-      <c r="H51" s="11" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="52" spans="8:8" x14ac:dyDescent="0.3">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="51" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="H51" s="9" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="52" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B52" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="C52" s="12"/>
+      <c r="D52" s="12"/>
       <c r="H52" s="8" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="53" spans="8:8" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="53" spans="2:14" x14ac:dyDescent="0.3">
       <c r="H53" s="6"/>
     </row>
-    <row r="54" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B54" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D54" s="5" t="s">
+        <v>7</v>
+      </c>
       <c r="H54" s="6"/>
     </row>
-    <row r="55" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B55" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="D55" s="4"/>
       <c r="H55" s="6"/>
     </row>
+    <row r="56" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B56" s="12"/>
+      <c r="D56" s="4"/>
+    </row>
+    <row r="57" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B57" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D57" s="4"/>
+    </row>
+    <row r="58" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B58" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="L58" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="M58" s="12"/>
+      <c r="N58" s="12"/>
+    </row>
+    <row r="59" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B59" s="12"/>
+      <c r="F59" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="G59" s="12"/>
+      <c r="H59" s="12"/>
+    </row>
+    <row r="60" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B60" s="12"/>
+      <c r="D60" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="L60" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="N60" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="61" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B61" s="12"/>
+      <c r="D61" s="4"/>
+      <c r="F61" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H61" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="L61" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="N61" s="4"/>
+    </row>
+    <row r="62" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B62" s="12"/>
+      <c r="D62" s="4"/>
+      <c r="F62" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="H62" s="4"/>
+      <c r="L62" s="13"/>
+      <c r="N62" s="4"/>
+    </row>
+    <row r="63" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B63" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D63" s="4"/>
+      <c r="F63" s="12"/>
+      <c r="H63" s="4"/>
+      <c r="L63" s="2"/>
+      <c r="N63" s="4"/>
+    </row>
+    <row r="64" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B64" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D64" s="4"/>
+      <c r="F64" s="2"/>
+      <c r="H64" s="4"/>
+      <c r="L64" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="65" spans="2:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B65" s="14"/>
+      <c r="D65" s="4"/>
+      <c r="F65" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="L65" s="13" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="66" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B66" s="14"/>
+      <c r="D66" s="4"/>
+      <c r="F66" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="L66" s="13"/>
+      <c r="N66" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="67" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B67" s="14"/>
+      <c r="D67" s="4"/>
+      <c r="F67" s="12"/>
+      <c r="H67" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="L67" s="13"/>
+      <c r="N67" s="4"/>
+    </row>
+    <row r="68" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B68" s="14"/>
+      <c r="D68" s="4"/>
+      <c r="F68" s="12"/>
+      <c r="H68" s="4"/>
+      <c r="L68" s="13"/>
+      <c r="N68" s="4"/>
+    </row>
+    <row r="69" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B69" s="14"/>
+      <c r="D69" s="4"/>
+      <c r="F69" s="12"/>
+      <c r="H69" s="4"/>
+      <c r="L69" s="13"/>
+      <c r="N69" s="4"/>
+    </row>
+    <row r="70" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B70" s="14"/>
+      <c r="D70" s="4"/>
+      <c r="F70" s="12"/>
+      <c r="H70" s="4"/>
+      <c r="L70" s="2"/>
+      <c r="N70" s="4"/>
+    </row>
+    <row r="71" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B71" s="14"/>
+      <c r="D71" s="4"/>
+      <c r="F71" s="2"/>
+      <c r="H71" s="4"/>
+      <c r="L71" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="N71" s="4"/>
+    </row>
+    <row r="72" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="D72" s="4"/>
+      <c r="F72" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H72" s="4"/>
+      <c r="L72" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="N72" s="4"/>
+    </row>
+    <row r="73" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="D73" s="4"/>
+      <c r="F73" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="H73" s="4"/>
+      <c r="L73" s="13"/>
+      <c r="N73" s="4"/>
+    </row>
+    <row r="74" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="D74" s="4"/>
+      <c r="F74" s="12"/>
+      <c r="H74" s="4"/>
+      <c r="L74" s="13"/>
+      <c r="N74" s="4"/>
+    </row>
+    <row r="75" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="D75" s="4"/>
+      <c r="F75" s="12"/>
+      <c r="H75" s="4"/>
+      <c r="L75" s="13"/>
+      <c r="N75" s="4"/>
+    </row>
+    <row r="76" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="D76" s="4"/>
+      <c r="F76" s="12"/>
+      <c r="H76" s="4"/>
+      <c r="L76" s="14"/>
+      <c r="N76" s="4"/>
+    </row>
+    <row r="77" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="D77" s="4"/>
+      <c r="F77" s="14"/>
+      <c r="H77" s="4"/>
+      <c r="L77" s="14"/>
+      <c r="N77" s="4"/>
+    </row>
+    <row r="78" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="D78" s="4"/>
+      <c r="F78" s="14"/>
+      <c r="H78" s="4"/>
+      <c r="N78" s="4"/>
+    </row>
+    <row r="79" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="H79" s="4"/>
+      <c r="N79" s="4"/>
+    </row>
+    <row r="80" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="H80" s="4"/>
+      <c r="N80" s="4"/>
+    </row>
+    <row r="81" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="H81" s="4"/>
+      <c r="N81" s="4"/>
+    </row>
+    <row r="82" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="H82" s="4"/>
+      <c r="N82" s="4"/>
+    </row>
+    <row r="83" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="D83" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H83" s="4"/>
+      <c r="N83" s="4"/>
+    </row>
+    <row r="84" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="D84" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="H84" s="4"/>
+      <c r="N84" s="4"/>
+    </row>
+    <row r="85" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="D85" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="H85" s="4"/>
+      <c r="N85" s="4"/>
+    </row>
+    <row r="86" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="D86" s="6"/>
+      <c r="N86" s="4"/>
+    </row>
+    <row r="87" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="D87" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="N87" s="4"/>
+    </row>
+    <row r="88" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="D88" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="N88" s="4"/>
+    </row>
+    <row r="89" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="D89" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="N89" s="4"/>
+    </row>
+    <row r="90" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="D90" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="H90" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N90" s="4"/>
+    </row>
+    <row r="91" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="D91" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="H91" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="N91" s="4"/>
+    </row>
+    <row r="92" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="D92" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="H92" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="N92" s="4"/>
+    </row>
+    <row r="93" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="D93" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="H93" s="6"/>
+      <c r="N93" s="4"/>
+    </row>
+    <row r="94" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="D94" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="H94" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="N94" s="4"/>
+    </row>
+    <row r="95" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="D95" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="H95" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="N95" s="4"/>
+    </row>
+    <row r="96" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="D96" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="H96" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="N96" s="4"/>
+    </row>
+    <row r="97" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="D97" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="H97" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="N97" s="4"/>
+    </row>
+    <row r="98" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="D98" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="H98" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="N98" s="4"/>
+    </row>
+    <row r="99" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="D99" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="H99" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="N99" s="4"/>
+    </row>
+    <row r="100" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="H100" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="N100" s="4"/>
+    </row>
+    <row r="101" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="H101" s="8" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="102" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="H102" s="8" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="103" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="H103" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="N103" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="104" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="H104" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="N104" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="105" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="H105" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="N105" s="15" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="106" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="H106" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="N106" s="6"/>
+    </row>
+    <row r="107" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="N107" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="108" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="N108" s="8" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="109" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="N109" s="8" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="110" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="N110" s="8" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="111" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="N111" s="8" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="112" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="N112" s="8" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="113" spans="14:14" x14ac:dyDescent="0.3">
+      <c r="N113" s="8" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="114" spans="14:14" x14ac:dyDescent="0.3">
+      <c r="N114" s="8" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="115" spans="14:14" x14ac:dyDescent="0.3">
+      <c r="N115" s="8" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="116" spans="14:14" x14ac:dyDescent="0.3">
+      <c r="N116" s="8" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="117" spans="14:14" x14ac:dyDescent="0.3">
+      <c r="N117" s="8" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="118" spans="14:14" x14ac:dyDescent="0.3">
+      <c r="N118" s="8" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="119" spans="14:14" x14ac:dyDescent="0.3">
+      <c r="N119" s="8" t="s">
+        <v>94</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="16">
+    <mergeCell ref="F66:F70"/>
+    <mergeCell ref="F73:F76"/>
+    <mergeCell ref="L58:N58"/>
+    <mergeCell ref="L61:L62"/>
+    <mergeCell ref="L65:L69"/>
+    <mergeCell ref="L72:L75"/>
+    <mergeCell ref="B52:D52"/>
+    <mergeCell ref="B55:B56"/>
+    <mergeCell ref="B58:B62"/>
+    <mergeCell ref="F59:H59"/>
+    <mergeCell ref="F62:F63"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="F4:H4"/>
     <mergeCell ref="J4:L4"/>
@@ -3676,9 +6478,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{86e23165-d923-4ef0-ae5f-fd5f4d5ec307}" enabled="1" method="Standard" siteId="{eeb14196-63dc-45aa-ac42-0a4583b12590}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
Adición de pasos de ETL
</commit_message>
<xml_diff>
--- a/Segundo entregable/PlantillaDisenioETL.xlsx
+++ b/Segundo entregable/PlantillaDisenioETL.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fabrizio.cucina\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/fc549774c6d51506/Desktop/Ciencia de Datos/MIAD/3. Semestre III/5. ETL/IV Week IV/entrega_proyecto_MIAD_modelado_datos/Segundo entregable/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2B29A92-6E2A-4A43-AFE0-13C1E8EBAA8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{D2B29A92-6E2A-4A43-AFE0-13C1E8EBAA8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30A8371A-F583-45FE-BF45-255D8D2FE4B7}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="96">
   <si>
     <t>Inspirada en el trabajo realizado por el Grupo Krusty_Brand202214</t>
   </si>
@@ -335,6 +335,9 @@
   </si>
   <si>
     <t>ConteoOfertaBeneficio</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -441,19 +444,19 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2973,15 +2976,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>1562100</xdr:colOff>
-      <xdr:row>40</xdr:row>
+      <xdr:colOff>1517529</xdr:colOff>
+      <xdr:row>45</xdr:row>
       <xdr:rowOff>15240</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>1565910</xdr:colOff>
-      <xdr:row>44</xdr:row>
-      <xdr:rowOff>137160</xdr:rowOff>
+      <xdr:colOff>1524000</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>133048</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -2995,9 +2998,9 @@
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
-        <a:xfrm flipH="1">
-          <a:off x="12367260" y="7330440"/>
-          <a:ext cx="3810" cy="853440"/>
+        <a:xfrm>
+          <a:off x="12330672" y="8179526"/>
+          <a:ext cx="6471" cy="299236"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -3026,15 +3029,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>1790700</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
+      <xdr:colOff>1826986</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>12397</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>1798321</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>30480</xdr:rowOff>
+      <xdr:colOff>1834607</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>90955</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -3049,8 +3052,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="19362420" y="4522470"/>
-          <a:ext cx="7621" cy="445770"/>
+          <a:off x="19413462" y="5636683"/>
+          <a:ext cx="7621" cy="441415"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -3637,15 +3640,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1821180</xdr:colOff>
-      <xdr:row>77</xdr:row>
-      <xdr:rowOff>144780</xdr:rowOff>
+      <xdr:colOff>1772798</xdr:colOff>
+      <xdr:row>83</xdr:row>
+      <xdr:rowOff>24190</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1824990</xdr:colOff>
-      <xdr:row>81</xdr:row>
-      <xdr:rowOff>167640</xdr:rowOff>
+      <xdr:colOff>1790095</xdr:colOff>
+      <xdr:row>86</xdr:row>
+      <xdr:rowOff>155544</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -3660,8 +3663,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="5364480" y="5448300"/>
-          <a:ext cx="3810" cy="754380"/>
+          <a:off x="5316703" y="15082761"/>
+          <a:ext cx="17297" cy="675640"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -5079,6 +5082,257 @@
             </a:rPr>
             <a:t>T8. Calcular ConteoOfertaBeneficio = 1 por fila (para conteos distintos).</a:t>
           </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>169332</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>36286</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>2963333</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>84667</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="Rectángulo redondeado 20">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5DB03EE9-E495-46BF-9A1A-C01CCA0DCEC2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10982475" y="7293429"/>
+          <a:ext cx="2794001" cy="774095"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T6.</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100" b="0" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t> Validar consistencia y contenido de los datos de variables. </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr kumimoji="0" lang="es-CO" sz="1100" b="0" i="0" u="none" strike="noStrike" kern="0" cap="none" spc="0" normalizeH="0" baseline="0" noProof="0">
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:uLnTx/>
+              <a:uFillTx/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Así como mispelling en los mismos planes y servicios.</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-CO" sz="1100">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>92166</xdr:colOff>
+      <xdr:row>76</xdr:row>
+      <xdr:rowOff>1694</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>3597366</xdr:colOff>
+      <xdr:row>78</xdr:row>
+      <xdr:rowOff>169334</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="33" name="Rectángulo redondeado 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B70FA98E-81C1-484F-8E9A-68CEAB79CE9E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3636071" y="13790265"/>
+          <a:ext cx="3505200" cy="530498"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T6.</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t> Validar consistencia y contenido. Eliminar mispelling en los estados, condados.</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-CO" sz="1100">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>87328</xdr:colOff>
+      <xdr:row>79</xdr:row>
+      <xdr:rowOff>81523</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>3592528</xdr:colOff>
+      <xdr:row>82</xdr:row>
+      <xdr:rowOff>67735</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="69" name="Rectángulo redondeado 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C2D4A8FD-36EC-4205-9894-B237B0B93A3C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3631233" y="14414380"/>
+          <a:ext cx="3505200" cy="530498"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>T7.</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t> Verificar que el área de las pabolaciones es consistentes entre los condados.</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-CO" sz="1100">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </a:endParaRPr>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -5418,45 +5672,45 @@
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
-      <c r="J2" s="11"/>
-      <c r="K2" s="11"/>
-      <c r="L2" s="11"/>
-      <c r="M2" s="11"/>
-      <c r="N2" s="11"/>
-      <c r="O2" s="11"/>
-      <c r="P2" s="11"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="15"/>
+      <c r="L2" s="15"/>
+      <c r="M2" s="15"/>
+      <c r="N2" s="15"/>
+      <c r="O2" s="15"/>
+      <c r="P2" s="15"/>
     </row>
     <row r="4" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="F4" s="10" t="s">
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="F4" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-      <c r="J4" s="10" t="s">
+      <c r="G4" s="14"/>
+      <c r="H4" s="14"/>
+      <c r="J4" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="10"/>
-      <c r="L4" s="10"/>
-      <c r="N4" s="10" t="s">
+      <c r="K4" s="14"/>
+      <c r="L4" s="14"/>
+      <c r="N4" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="O4" s="10"/>
-      <c r="P4" s="10"/>
+      <c r="O4" s="14"/>
+      <c r="P4" s="14"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
@@ -5786,61 +6040,50 @@
     <row r="26" spans="2:16" x14ac:dyDescent="0.3">
       <c r="D26" s="4"/>
       <c r="H26" s="4"/>
+      <c r="L26" s="4"/>
       <c r="P26" s="6"/>
     </row>
     <row r="27" spans="2:16" x14ac:dyDescent="0.3">
       <c r="D27" s="4"/>
       <c r="H27" s="4"/>
+      <c r="L27" s="4"/>
       <c r="P27" s="6"/>
     </row>
     <row r="28" spans="2:16" x14ac:dyDescent="0.3">
       <c r="D28" s="4"/>
       <c r="H28" s="4"/>
-      <c r="L28" s="5" t="s">
-        <v>36</v>
-      </c>
+      <c r="L28" s="4"/>
       <c r="P28" s="6"/>
     </row>
     <row r="29" spans="2:16" x14ac:dyDescent="0.3">
       <c r="D29" s="4"/>
       <c r="H29" s="4"/>
-      <c r="L29" s="6" t="s">
-        <v>37</v>
-      </c>
+      <c r="L29" s="4"/>
       <c r="P29" s="6"/>
     </row>
     <row r="30" spans="2:16" x14ac:dyDescent="0.3">
       <c r="D30" s="4"/>
       <c r="H30" s="4"/>
-      <c r="L30" s="8" t="s">
-        <v>38</v>
-      </c>
+      <c r="L30" s="4"/>
       <c r="P30" s="6"/>
     </row>
     <row r="31" spans="2:16" x14ac:dyDescent="0.3">
       <c r="H31" s="4"/>
-      <c r="L31" s="6"/>
       <c r="P31" s="6"/>
     </row>
     <row r="32" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="F32" t="s">
+        <v>95</v>
+      </c>
       <c r="H32" s="4"/>
-      <c r="L32" s="6" t="s">
-        <v>39</v>
-      </c>
       <c r="P32" s="6"/>
     </row>
     <row r="33" spans="4:16" x14ac:dyDescent="0.3">
       <c r="H33" s="4"/>
-      <c r="L33" s="9" t="s">
-        <v>40</v>
-      </c>
       <c r="P33" s="6"/>
     </row>
     <row r="34" spans="4:16" x14ac:dyDescent="0.3">
       <c r="H34" s="4"/>
-      <c r="L34" s="8" t="s">
-        <v>14</v>
-      </c>
       <c r="P34" s="6"/>
     </row>
     <row r="35" spans="4:16" x14ac:dyDescent="0.3">
@@ -5848,6 +6091,9 @@
         <v>36</v>
       </c>
       <c r="H35" s="4"/>
+      <c r="L35" s="5" t="s">
+        <v>36</v>
+      </c>
       <c r="P35" s="6"/>
     </row>
     <row r="36" spans="4:16" x14ac:dyDescent="0.3">
@@ -5855,6 +6101,9 @@
         <v>37</v>
       </c>
       <c r="H36" s="4"/>
+      <c r="L36" s="6" t="s">
+        <v>37</v>
+      </c>
       <c r="P36" s="7"/>
     </row>
     <row r="37" spans="4:16" x14ac:dyDescent="0.3">
@@ -5862,11 +6111,15 @@
         <v>41</v>
       </c>
       <c r="H37" s="4"/>
+      <c r="L37" s="8" t="s">
+        <v>38</v>
+      </c>
       <c r="P37" s="7"/>
     </row>
     <row r="38" spans="4:16" x14ac:dyDescent="0.3">
       <c r="D38" s="6"/>
       <c r="H38" s="4"/>
+      <c r="L38" s="6"/>
       <c r="P38" s="5" t="s">
         <v>36</v>
       </c>
@@ -5876,6 +6129,9 @@
         <v>39</v>
       </c>
       <c r="H39" s="4"/>
+      <c r="L39" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="P39" s="6" t="s">
         <v>37</v>
       </c>
@@ -5885,6 +6141,9 @@
         <v>42</v>
       </c>
       <c r="H40" s="4"/>
+      <c r="L40" s="9" t="s">
+        <v>40</v>
+      </c>
       <c r="P40" s="8" t="s">
         <v>43</v>
       </c>
@@ -5894,12 +6153,16 @@
         <v>12</v>
       </c>
       <c r="H41" s="4"/>
+      <c r="L41" s="8" t="s">
+        <v>14</v>
+      </c>
       <c r="P41" s="6"/>
     </row>
     <row r="42" spans="4:16" x14ac:dyDescent="0.3">
       <c r="D42" s="8" t="s">
         <v>44</v>
       </c>
+      <c r="H42" s="4"/>
       <c r="P42" s="6" t="s">
         <v>39</v>
       </c>
@@ -5908,6 +6171,7 @@
       <c r="D43" s="8" t="s">
         <v>45</v>
       </c>
+      <c r="H43" s="4"/>
       <c r="P43" s="9" t="s">
         <v>15</v>
       </c>
@@ -5916,6 +6180,7 @@
       <c r="D44" s="8" t="s">
         <v>46</v>
       </c>
+      <c r="H44" s="4"/>
       <c r="P44" s="8" t="s">
         <v>17</v>
       </c>
@@ -5924,6 +6189,7 @@
       <c r="D45" s="8" t="s">
         <v>47</v>
       </c>
+      <c r="H45" s="4"/>
       <c r="P45" s="9" t="s">
         <v>20</v>
       </c>
@@ -5932,45 +6198,39 @@
       <c r="D46" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="H46" s="5" t="s">
+    </row>
+    <row r="48" spans="4:16" x14ac:dyDescent="0.3">
+      <c r="H48" s="5" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="47" spans="4:16" x14ac:dyDescent="0.3">
-      <c r="H47" s="6" t="s">
+    <row r="49" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="H49" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="48" spans="4:16" x14ac:dyDescent="0.3">
-      <c r="H48" s="8" t="s">
+    <row r="50" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="H50" s="8" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="49" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="H49" s="6"/>
-    </row>
-    <row r="50" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="H50" s="6" t="s">
+    <row r="51" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="H51" s="6"/>
+    </row>
+    <row r="52" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B52" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="C52" s="13"/>
+      <c r="D52" s="13"/>
+      <c r="H52" s="6" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="51" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="H51" s="9" t="s">
+    <row r="53" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="H53" s="9" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="52" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B52" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="C52" s="12"/>
-      <c r="D52" s="12"/>
-      <c r="H52" s="8" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="53" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="H53" s="6"/>
     </row>
     <row r="54" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B54" s="3" t="s">
@@ -5979,45 +6239,49 @@
       <c r="D54" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="H54" s="6"/>
+      <c r="H54" s="8" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="55" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B55" s="13" t="s">
+      <c r="B55" s="12" t="s">
         <v>53</v>
       </c>
       <c r="D55" s="4"/>
       <c r="H55" s="6"/>
     </row>
     <row r="56" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B56" s="12"/>
+      <c r="B56" s="13"/>
       <c r="D56" s="4"/>
+      <c r="H56" s="6"/>
     </row>
     <row r="57" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B57" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D57" s="4"/>
+      <c r="H57" s="6"/>
     </row>
     <row r="58" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B58" s="13" t="s">
+      <c r="B58" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="L58" s="10" t="s">
+      <c r="L58" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="M58" s="12"/>
-      <c r="N58" s="12"/>
+      <c r="M58" s="13"/>
+      <c r="N58" s="13"/>
     </row>
     <row r="59" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B59" s="12"/>
-      <c r="F59" s="10" t="s">
+      <c r="B59" s="13"/>
+      <c r="F59" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="G59" s="12"/>
-      <c r="H59" s="12"/>
+      <c r="G59" s="13"/>
+      <c r="H59" s="13"/>
     </row>
     <row r="60" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B60" s="12"/>
+      <c r="B60" s="13"/>
       <c r="D60" s="5" t="s">
         <v>18</v>
       </c>
@@ -6029,7 +6293,7 @@
       </c>
     </row>
     <row r="61" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B61" s="12"/>
+      <c r="B61" s="13"/>
       <c r="D61" s="4"/>
       <c r="F61" s="3" t="s">
         <v>6</v>
@@ -6037,19 +6301,19 @@
       <c r="H61" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="L61" s="13" t="s">
+      <c r="L61" s="12" t="s">
         <v>83</v>
       </c>
       <c r="N61" s="4"/>
     </row>
     <row r="62" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B62" s="12"/>
+      <c r="B62" s="13"/>
       <c r="D62" s="4"/>
-      <c r="F62" s="13" t="s">
+      <c r="F62" s="12" t="s">
         <v>10</v>
       </c>
       <c r="H62" s="4"/>
-      <c r="L62" s="13"/>
+      <c r="L62" s="12"/>
       <c r="N62" s="4"/>
     </row>
     <row r="63" spans="2:14" x14ac:dyDescent="0.3">
@@ -6057,7 +6321,7 @@
         <v>19</v>
       </c>
       <c r="D63" s="4"/>
-      <c r="F63" s="12"/>
+      <c r="F63" s="13"/>
       <c r="H63" s="4"/>
       <c r="L63" s="2"/>
       <c r="N63" s="4"/>
@@ -6074,62 +6338,62 @@
       </c>
     </row>
     <row r="65" spans="2:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B65" s="14"/>
+      <c r="B65" s="10"/>
       <c r="D65" s="4"/>
       <c r="F65" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="L65" s="13" t="s">
+      <c r="L65" s="12" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="66" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B66" s="14"/>
+      <c r="B66" s="10"/>
       <c r="D66" s="4"/>
-      <c r="F66" s="13" t="s">
+      <c r="F66" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="L66" s="13"/>
+      <c r="L66" s="12"/>
       <c r="N66" s="5" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="67" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B67" s="14"/>
+      <c r="B67" s="10"/>
       <c r="D67" s="4"/>
-      <c r="F67" s="12"/>
+      <c r="F67" s="13"/>
       <c r="H67" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="L67" s="13"/>
+      <c r="L67" s="12"/>
       <c r="N67" s="4"/>
     </row>
     <row r="68" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B68" s="14"/>
+      <c r="B68" s="10"/>
       <c r="D68" s="4"/>
-      <c r="F68" s="12"/>
+      <c r="F68" s="13"/>
       <c r="H68" s="4"/>
-      <c r="L68" s="13"/>
+      <c r="L68" s="12"/>
       <c r="N68" s="4"/>
     </row>
     <row r="69" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B69" s="14"/>
+      <c r="B69" s="10"/>
       <c r="D69" s="4"/>
-      <c r="F69" s="12"/>
+      <c r="F69" s="13"/>
       <c r="H69" s="4"/>
-      <c r="L69" s="13"/>
+      <c r="L69" s="12"/>
       <c r="N69" s="4"/>
     </row>
     <row r="70" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B70" s="14"/>
+      <c r="B70" s="10"/>
       <c r="D70" s="4"/>
-      <c r="F70" s="12"/>
+      <c r="F70" s="13"/>
       <c r="H70" s="4"/>
       <c r="L70" s="2"/>
       <c r="N70" s="4"/>
     </row>
     <row r="71" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B71" s="14"/>
+      <c r="B71" s="10"/>
       <c r="D71" s="4"/>
       <c r="F71" s="2"/>
       <c r="H71" s="4"/>
@@ -6144,116 +6408,108 @@
         <v>19</v>
       </c>
       <c r="H72" s="4"/>
-      <c r="L72" s="13" t="s">
+      <c r="L72" s="12" t="s">
         <v>71</v>
       </c>
       <c r="N72" s="4"/>
     </row>
     <row r="73" spans="2:14" x14ac:dyDescent="0.3">
       <c r="D73" s="4"/>
-      <c r="F73" s="13" t="s">
+      <c r="F73" s="12" t="s">
         <v>71</v>
       </c>
       <c r="H73" s="4"/>
-      <c r="L73" s="13"/>
+      <c r="L73" s="12"/>
       <c r="N73" s="4"/>
     </row>
     <row r="74" spans="2:14" x14ac:dyDescent="0.3">
       <c r="D74" s="4"/>
-      <c r="F74" s="12"/>
+      <c r="F74" s="13"/>
       <c r="H74" s="4"/>
-      <c r="L74" s="13"/>
+      <c r="L74" s="12"/>
       <c r="N74" s="4"/>
     </row>
     <row r="75" spans="2:14" x14ac:dyDescent="0.3">
       <c r="D75" s="4"/>
-      <c r="F75" s="12"/>
+      <c r="F75" s="13"/>
       <c r="H75" s="4"/>
-      <c r="L75" s="13"/>
+      <c r="L75" s="12"/>
       <c r="N75" s="4"/>
     </row>
     <row r="76" spans="2:14" x14ac:dyDescent="0.3">
       <c r="D76" s="4"/>
-      <c r="F76" s="12"/>
+      <c r="F76" s="13"/>
       <c r="H76" s="4"/>
-      <c r="L76" s="14"/>
+      <c r="L76" s="10"/>
       <c r="N76" s="4"/>
     </row>
     <row r="77" spans="2:14" x14ac:dyDescent="0.3">
       <c r="D77" s="4"/>
-      <c r="F77" s="14"/>
+      <c r="F77" s="10"/>
       <c r="H77" s="4"/>
-      <c r="L77" s="14"/>
+      <c r="L77" s="10"/>
       <c r="N77" s="4"/>
     </row>
     <row r="78" spans="2:14" x14ac:dyDescent="0.3">
       <c r="D78" s="4"/>
-      <c r="F78" s="14"/>
+      <c r="F78" s="10"/>
       <c r="H78" s="4"/>
       <c r="N78" s="4"/>
     </row>
     <row r="79" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="D79" s="4"/>
       <c r="H79" s="4"/>
       <c r="N79" s="4"/>
     </row>
     <row r="80" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="D80" s="4"/>
       <c r="H80" s="4"/>
       <c r="N80" s="4"/>
     </row>
     <row r="81" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="D81" s="4"/>
       <c r="H81" s="4"/>
       <c r="N81" s="4"/>
     </row>
     <row r="82" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="D82" s="4"/>
       <c r="H82" s="4"/>
       <c r="N82" s="4"/>
     </row>
     <row r="83" spans="4:14" x14ac:dyDescent="0.3">
-      <c r="D83" s="5" t="s">
-        <v>36</v>
-      </c>
+      <c r="D83" s="4"/>
       <c r="H83" s="4"/>
       <c r="N83" s="4"/>
     </row>
     <row r="84" spans="4:14" x14ac:dyDescent="0.3">
-      <c r="D84" s="6" t="s">
-        <v>37</v>
-      </c>
       <c r="H84" s="4"/>
       <c r="N84" s="4"/>
     </row>
     <row r="85" spans="4:14" x14ac:dyDescent="0.3">
-      <c r="D85" s="8" t="s">
-        <v>56</v>
-      </c>
       <c r="H85" s="4"/>
       <c r="N85" s="4"/>
     </row>
     <row r="86" spans="4:14" x14ac:dyDescent="0.3">
-      <c r="D86" s="6"/>
       <c r="N86" s="4"/>
     </row>
     <row r="87" spans="4:14" x14ac:dyDescent="0.3">
-      <c r="D87" s="6" t="s">
-        <v>39</v>
-      </c>
       <c r="N87" s="4"/>
     </row>
     <row r="88" spans="4:14" x14ac:dyDescent="0.3">
-      <c r="D88" s="8" t="s">
-        <v>68</v>
+      <c r="D88" s="5" t="s">
+        <v>36</v>
       </c>
       <c r="N88" s="4"/>
     </row>
     <row r="89" spans="4:14" x14ac:dyDescent="0.3">
-      <c r="D89" s="8" t="s">
-        <v>57</v>
+      <c r="D89" s="6" t="s">
+        <v>37</v>
       </c>
       <c r="N89" s="4"/>
     </row>
     <row r="90" spans="4:14" x14ac:dyDescent="0.3">
       <c r="D90" s="8" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H90" s="5" t="s">
         <v>36</v>
@@ -6261,33 +6517,31 @@
       <c r="N90" s="4"/>
     </row>
     <row r="91" spans="4:14" x14ac:dyDescent="0.3">
-      <c r="D91" s="8" t="s">
-        <v>59</v>
-      </c>
+      <c r="D91" s="6"/>
       <c r="H91" s="6" t="s">
         <v>37</v>
       </c>
       <c r="N91" s="4"/>
     </row>
     <row r="92" spans="4:14" x14ac:dyDescent="0.3">
-      <c r="D92" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="H92" s="15" t="s">
+      <c r="D92" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="H92" s="11" t="s">
         <v>72</v>
       </c>
       <c r="N92" s="4"/>
     </row>
     <row r="93" spans="4:14" x14ac:dyDescent="0.3">
       <c r="D93" s="8" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="H93" s="6"/>
       <c r="N93" s="4"/>
     </row>
     <row r="94" spans="4:14" x14ac:dyDescent="0.3">
       <c r="D94" s="8" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="H94" s="6" t="s">
         <v>39</v>
@@ -6296,7 +6550,7 @@
     </row>
     <row r="95" spans="4:14" x14ac:dyDescent="0.3">
       <c r="D95" s="8" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="H95" s="8" t="s">
         <v>73</v>
@@ -6305,7 +6559,7 @@
     </row>
     <row r="96" spans="4:14" x14ac:dyDescent="0.3">
       <c r="D96" s="8" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="H96" s="8" t="s">
         <v>74</v>
@@ -6314,7 +6568,7 @@
     </row>
     <row r="97" spans="4:14" x14ac:dyDescent="0.3">
       <c r="D97" s="8" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="H97" s="8" t="s">
         <v>75</v>
@@ -6323,7 +6577,7 @@
     </row>
     <row r="98" spans="4:14" x14ac:dyDescent="0.3">
       <c r="D98" s="8" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="H98" s="8" t="s">
         <v>76</v>
@@ -6332,7 +6586,7 @@
     </row>
     <row r="99" spans="4:14" x14ac:dyDescent="0.3">
       <c r="D99" s="8" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="H99" s="8" t="s">
         <v>77</v>
@@ -6340,22 +6594,34 @@
       <c r="N99" s="4"/>
     </row>
     <row r="100" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="D100" s="8" t="s">
+        <v>63</v>
+      </c>
       <c r="H100" s="8" t="s">
         <v>78</v>
       </c>
       <c r="N100" s="4"/>
     </row>
     <row r="101" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="D101" s="8" t="s">
+        <v>64</v>
+      </c>
       <c r="H101" s="8" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="102" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="D102" s="8" t="s">
+        <v>65</v>
+      </c>
       <c r="H102" s="8" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="103" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="D103" s="8" t="s">
+        <v>66</v>
+      </c>
       <c r="H103" s="8" t="s">
         <v>81</v>
       </c>
@@ -6364,6 +6630,9 @@
       </c>
     </row>
     <row r="104" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="D104" s="8" t="s">
+        <v>67</v>
+      </c>
       <c r="H104" s="8" t="s">
         <v>65</v>
       </c>
@@ -6375,7 +6644,7 @@
       <c r="H105" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="N105" s="15" t="s">
+      <c r="N105" s="11" t="s">
         <v>82</v>
       </c>
     </row>
@@ -6452,22 +6721,22 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="N4:P4"/>
+    <mergeCell ref="B2:P2"/>
+    <mergeCell ref="B52:D52"/>
+    <mergeCell ref="B55:B56"/>
+    <mergeCell ref="B58:B62"/>
+    <mergeCell ref="F59:H59"/>
+    <mergeCell ref="F62:F63"/>
     <mergeCell ref="F66:F70"/>
     <mergeCell ref="F73:F76"/>
     <mergeCell ref="L58:N58"/>
     <mergeCell ref="L61:L62"/>
     <mergeCell ref="L65:L69"/>
     <mergeCell ref="L72:L75"/>
-    <mergeCell ref="B52:D52"/>
-    <mergeCell ref="B55:B56"/>
-    <mergeCell ref="B58:B62"/>
-    <mergeCell ref="F59:H59"/>
-    <mergeCell ref="F62:F63"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="F4:H4"/>
-    <mergeCell ref="J4:L4"/>
-    <mergeCell ref="N4:P4"/>
-    <mergeCell ref="B2:P2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>

</xml_diff>